<commit_message>
change the structure, fix a lot of stuff, add a new report
</commit_message>
<xml_diff>
--- a/Mil.Paperwork.Domain/Templates/ResidualValueReportTemplate.xlsx
+++ b/Mil.Paperwork.Domain/Templates/ResidualValueReportTemplate.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\Projects\Mil.Paperwork.WriteOff\Mil.Paperwork.Domain\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45E1B699-A6AB-4C5E-B963-C8CF80867B06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7E80A4F-BCC2-4309-9075-5A94E82FA98C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Відомість" sheetId="1" r:id="rId1"/>
@@ -68,9 +68,6 @@
   </si>
   <si>
     <t>ЗАТВЕРДЖУЮ</t>
-  </si>
-  <si>
-    <t>"____" __________ 2025 року</t>
   </si>
   <si>
     <t>ВІДОМІСТЬ</t>
@@ -303,6 +300,9 @@
   </si>
   <si>
     <t>Командир військової частини [MIL_UNIT]</t>
+  </si>
+  <si>
+    <t>"____" __________ 2026 року</t>
   </si>
 </sst>
 </file>
@@ -1119,13 +1119,62 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1149,57 +1198,8 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1924,24 +1924,24 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:Y1003"/>
-  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="8.54296875" style="6" customWidth="1"/>
-    <col min="2" max="2" width="40.1796875" style="6" customWidth="1"/>
-    <col min="3" max="3" width="8.6328125" style="6" customWidth="1"/>
-    <col min="4" max="4" width="9.81640625" style="6" customWidth="1"/>
-    <col min="5" max="5" width="24.36328125" style="6" customWidth="1"/>
-    <col min="6" max="6" width="13.36328125" style="6" customWidth="1"/>
-    <col min="7" max="7" width="12.26953125" style="6" customWidth="1"/>
-    <col min="8" max="8" width="18.81640625" style="6" customWidth="1"/>
-    <col min="9" max="11" width="7.7265625" style="6" customWidth="1"/>
-    <col min="12" max="13" width="14.453125" style="6" customWidth="1"/>
-    <col min="14" max="14" width="14.54296875" style="6" customWidth="1"/>
-    <col min="15" max="15" width="14.453125" style="6" customWidth="1"/>
-    <col min="16" max="25" width="13.26953125" style="6" customWidth="1"/>
-    <col min="26" max="998" width="14.453125" style="6"/>
-    <col min="999" max="9998" width="15.1796875" style="6" customWidth="1"/>
-    <col min="9999" max="16384" width="16.1796875" style="6" customWidth="1"/>
+    <col min="1" max="1" width="8.5546875" style="6" customWidth="1"/>
+    <col min="2" max="2" width="40.21875" style="6" customWidth="1"/>
+    <col min="3" max="3" width="8.6640625" style="6" customWidth="1"/>
+    <col min="4" max="4" width="9.77734375" style="6" customWidth="1"/>
+    <col min="5" max="5" width="24.33203125" style="6" customWidth="1"/>
+    <col min="6" max="6" width="13.33203125" style="6" customWidth="1"/>
+    <col min="7" max="7" width="12.21875" style="6" customWidth="1"/>
+    <col min="8" max="8" width="18.77734375" style="6" customWidth="1"/>
+    <col min="9" max="11" width="7.77734375" style="6" customWidth="1"/>
+    <col min="12" max="13" width="14.44140625" style="6" customWidth="1"/>
+    <col min="14" max="14" width="14.5546875" style="6" customWidth="1"/>
+    <col min="15" max="15" width="14.44140625" style="6" customWidth="1"/>
+    <col min="16" max="25" width="13.21875" style="6" customWidth="1"/>
+    <col min="26" max="998" width="14.44140625" style="6"/>
+    <col min="999" max="9998" width="15.21875" style="6" customWidth="1"/>
+    <col min="9999" max="16384" width="16.21875" style="6" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="12.75" customHeight="1">
@@ -1999,10 +1999,10 @@
       <c r="Y2" s="5"/>
     </row>
     <row r="3" spans="1:25" ht="12.75" customHeight="1">
-      <c r="A3" s="76" t="s">
-        <v>63</v>
+      <c r="A3" s="93" t="s">
+        <v>62</v>
       </c>
-      <c r="B3" s="77"/>
+      <c r="B3" s="94"/>
       <c r="C3" s="5"/>
       <c r="D3" s="5"/>
       <c r="E3" s="5"/>
@@ -2028,14 +2028,14 @@
       <c r="Y3" s="5"/>
     </row>
     <row r="4" spans="1:25" ht="12.75" customHeight="1">
-      <c r="A4" s="78" t="s">
+      <c r="A4" s="95" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="77"/>
-      <c r="C4" s="80" t="s">
-        <v>24</v>
+      <c r="B4" s="94"/>
+      <c r="C4" s="97" t="s">
+        <v>23</v>
       </c>
-      <c r="D4" s="81"/>
+      <c r="D4" s="98"/>
       <c r="E4" s="27"/>
       <c r="F4" s="5"/>
       <c r="G4" s="5"/>
@@ -2086,19 +2086,19 @@
       <c r="Y5" s="5"/>
     </row>
     <row r="6" spans="1:25" ht="18" customHeight="1">
-      <c r="A6" s="79"/>
-      <c r="B6" s="77"/>
+      <c r="A6" s="96"/>
+      <c r="B6" s="94"/>
       <c r="C6" s="7"/>
       <c r="D6" s="7"/>
       <c r="E6" s="7"/>
       <c r="F6" s="7"/>
-      <c r="K6" s="74" t="s">
+      <c r="K6" s="92" t="s">
         <v>1</v>
       </c>
-      <c r="L6" s="74"/>
-      <c r="M6" s="74"/>
-      <c r="N6" s="74"/>
-      <c r="O6" s="74"/>
+      <c r="L6" s="92"/>
+      <c r="M6" s="92"/>
+      <c r="N6" s="92"/>
+      <c r="O6" s="92"/>
       <c r="P6" s="20"/>
     </row>
     <row r="7" spans="1:25" ht="18">
@@ -2108,12 +2108,12 @@
       <c r="D7" s="7"/>
       <c r="E7" s="7"/>
       <c r="K7" s="75" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
-      <c r="L7" s="74"/>
-      <c r="M7" s="74"/>
-      <c r="N7" s="74"/>
-      <c r="O7" s="74"/>
+      <c r="L7" s="92"/>
+      <c r="M7" s="92"/>
+      <c r="N7" s="92"/>
+      <c r="O7" s="92"/>
       <c r="P7" s="20"/>
     </row>
     <row r="8" spans="1:25" ht="18" customHeight="1">
@@ -2122,15 +2122,15 @@
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
       <c r="E8" s="7"/>
-      <c r="K8" s="87" t="s">
+      <c r="K8" s="81" t="s">
+        <v>60</v>
+      </c>
+      <c r="L8" s="81"/>
+      <c r="M8" s="81"/>
+      <c r="N8" s="91" t="s">
         <v>61</v>
       </c>
-      <c r="L8" s="87"/>
-      <c r="M8" s="87"/>
-      <c r="N8" s="73" t="s">
-        <v>62</v>
-      </c>
-      <c r="O8" s="73"/>
+      <c r="O8" s="91"/>
       <c r="P8" s="8"/>
     </row>
     <row r="9" spans="1:25" ht="24.75" customHeight="1">
@@ -2139,13 +2139,13 @@
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
       <c r="E9" s="7"/>
-      <c r="K9" s="74" t="s">
-        <v>2</v>
+      <c r="K9" s="92" t="s">
+        <v>72</v>
       </c>
-      <c r="L9" s="74"/>
-      <c r="M9" s="74"/>
-      <c r="N9" s="74"/>
-      <c r="O9" s="74"/>
+      <c r="L9" s="92"/>
+      <c r="M9" s="92"/>
+      <c r="N9" s="92"/>
+      <c r="O9" s="92"/>
       <c r="P9" s="20"/>
     </row>
     <row r="10" spans="1:25" ht="18" customHeight="1">
@@ -2166,23 +2166,23 @@
       <c r="Y10" s="8"/>
     </row>
     <row r="11" spans="1:25" ht="18" customHeight="1">
-      <c r="A11" s="86" t="s">
-        <v>3</v>
+      <c r="A11" s="101" t="s">
+        <v>2</v>
       </c>
-      <c r="B11" s="86"/>
-      <c r="C11" s="86"/>
-      <c r="D11" s="86"/>
-      <c r="E11" s="86"/>
-      <c r="F11" s="86"/>
-      <c r="G11" s="86"/>
-      <c r="H11" s="86"/>
-      <c r="I11" s="86"/>
-      <c r="J11" s="86"/>
-      <c r="K11" s="86"/>
-      <c r="L11" s="86"/>
-      <c r="M11" s="86"/>
-      <c r="N11" s="86"/>
-      <c r="O11" s="86"/>
+      <c r="B11" s="101"/>
+      <c r="C11" s="101"/>
+      <c r="D11" s="101"/>
+      <c r="E11" s="101"/>
+      <c r="F11" s="101"/>
+      <c r="G11" s="101"/>
+      <c r="H11" s="101"/>
+      <c r="I11" s="101"/>
+      <c r="J11" s="101"/>
+      <c r="K11" s="101"/>
+      <c r="L11" s="101"/>
+      <c r="M11" s="101"/>
+      <c r="N11" s="101"/>
+      <c r="O11" s="101"/>
       <c r="P11" s="8"/>
       <c r="Q11" s="8"/>
       <c r="R11" s="8"/>
@@ -2195,87 +2195,87 @@
       <c r="Y11" s="8"/>
     </row>
     <row r="12" spans="1:25" ht="18" customHeight="1">
-      <c r="A12" s="83" t="s">
+      <c r="A12" s="100" t="s">
+        <v>32</v>
+      </c>
+      <c r="B12" s="100"/>
+      <c r="C12" s="100"/>
+      <c r="D12" s="100"/>
+      <c r="E12" s="100"/>
+      <c r="F12" s="100"/>
+      <c r="G12" s="100"/>
+      <c r="H12" s="100"/>
+      <c r="I12" s="100"/>
+      <c r="J12" s="100"/>
+      <c r="K12" s="100"/>
+      <c r="L12" s="100"/>
+      <c r="M12" s="100"/>
+      <c r="N12" s="100"/>
+      <c r="O12" s="100"/>
+      <c r="P12" s="8"/>
+    </row>
+    <row r="13" spans="1:25" s="37" customFormat="1" ht="18" customHeight="1">
+      <c r="A13" s="100" t="s">
+        <v>58</v>
+      </c>
+      <c r="B13" s="100"/>
+      <c r="C13" s="100"/>
+      <c r="D13" s="100"/>
+      <c r="E13" s="100"/>
+      <c r="F13" s="100"/>
+      <c r="G13" s="100"/>
+      <c r="H13" s="100"/>
+      <c r="I13" s="100"/>
+      <c r="J13" s="100"/>
+      <c r="K13" s="100"/>
+      <c r="L13" s="100"/>
+      <c r="M13" s="100"/>
+      <c r="N13" s="100"/>
+      <c r="O13" s="100"/>
+      <c r="P13" s="8"/>
+    </row>
+    <row r="14" spans="1:25" ht="18" customHeight="1">
+      <c r="A14" s="101"/>
+      <c r="B14" s="101"/>
+      <c r="C14" s="101"/>
+      <c r="D14" s="101"/>
+      <c r="E14" s="101"/>
+      <c r="F14" s="101"/>
+      <c r="G14" s="101"/>
+      <c r="H14" s="101"/>
+      <c r="I14" s="101"/>
+      <c r="J14" s="101"/>
+      <c r="K14" s="101"/>
+      <c r="L14" s="101"/>
+      <c r="M14" s="101"/>
+      <c r="N14" s="101"/>
+      <c r="O14" s="101"/>
+      <c r="P14" s="8"/>
+    </row>
+    <row r="15" spans="1:25" ht="67.95" customHeight="1">
+      <c r="A15" s="84" t="s">
+        <v>3</v>
+      </c>
+      <c r="B15" s="84" t="s">
+        <v>4</v>
+      </c>
+      <c r="C15" s="84" t="s">
+        <v>5</v>
+      </c>
+      <c r="D15" s="87" t="s">
+        <v>6</v>
+      </c>
+      <c r="E15" s="99" t="s">
         <v>33</v>
       </c>
-      <c r="B12" s="83"/>
-      <c r="C12" s="83"/>
-      <c r="D12" s="83"/>
-      <c r="E12" s="83"/>
-      <c r="F12" s="83"/>
-      <c r="G12" s="83"/>
-      <c r="H12" s="83"/>
-      <c r="I12" s="83"/>
-      <c r="J12" s="83"/>
-      <c r="K12" s="83"/>
-      <c r="L12" s="83"/>
-      <c r="M12" s="83"/>
-      <c r="N12" s="83"/>
-      <c r="O12" s="83"/>
-      <c r="P12" s="8"/>
-    </row>
-    <row r="13" spans="1:25" s="37" customFormat="1" ht="18" customHeight="1">
-      <c r="A13" s="83" t="s">
+      <c r="F15" s="89" t="s">
+        <v>21</v>
+      </c>
+      <c r="G15" s="84" t="s">
         <v>59</v>
       </c>
-      <c r="B13" s="83"/>
-      <c r="C13" s="83"/>
-      <c r="D13" s="83"/>
-      <c r="E13" s="83"/>
-      <c r="F13" s="83"/>
-      <c r="G13" s="83"/>
-      <c r="H13" s="83"/>
-      <c r="I13" s="83"/>
-      <c r="J13" s="83"/>
-      <c r="K13" s="83"/>
-      <c r="L13" s="83"/>
-      <c r="M13" s="83"/>
-      <c r="N13" s="83"/>
-      <c r="O13" s="83"/>
-      <c r="P13" s="8"/>
-    </row>
-    <row r="14" spans="1:25" ht="18" customHeight="1">
-      <c r="A14" s="86"/>
-      <c r="B14" s="86"/>
-      <c r="C14" s="86"/>
-      <c r="D14" s="86"/>
-      <c r="E14" s="86"/>
-      <c r="F14" s="86"/>
-      <c r="G14" s="86"/>
-      <c r="H14" s="86"/>
-      <c r="I14" s="86"/>
-      <c r="J14" s="86"/>
-      <c r="K14" s="86"/>
-      <c r="L14" s="86"/>
-      <c r="M14" s="86"/>
-      <c r="N14" s="86"/>
-      <c r="O14" s="86"/>
-      <c r="P14" s="8"/>
-    </row>
-    <row r="15" spans="1:25" ht="68" customHeight="1">
-      <c r="A15" s="84" t="s">
-        <v>4</v>
-      </c>
-      <c r="B15" s="84" t="s">
-        <v>5</v>
-      </c>
-      <c r="C15" s="84" t="s">
-        <v>6</v>
-      </c>
-      <c r="D15" s="91" t="s">
+      <c r="H15" s="82" t="s">
         <v>7</v>
-      </c>
-      <c r="E15" s="82" t="s">
-        <v>34</v>
-      </c>
-      <c r="F15" s="93" t="s">
-        <v>22</v>
-      </c>
-      <c r="G15" s="84" t="s">
-        <v>60</v>
-      </c>
-      <c r="H15" s="88" t="s">
-        <v>8</v>
       </c>
       <c r="I15" s="28"/>
       <c r="M15" s="28"/>
@@ -2283,14 +2283,14 @@
       <c r="O15" s="10"/>
     </row>
     <row r="16" spans="1:25" ht="24" customHeight="1">
-      <c r="A16" s="90"/>
-      <c r="B16" s="85"/>
-      <c r="C16" s="85"/>
-      <c r="D16" s="92"/>
-      <c r="E16" s="82"/>
-      <c r="F16" s="94"/>
-      <c r="G16" s="85"/>
-      <c r="H16" s="89"/>
+      <c r="A16" s="85"/>
+      <c r="B16" s="86"/>
+      <c r="C16" s="86"/>
+      <c r="D16" s="88"/>
+      <c r="E16" s="99"/>
+      <c r="F16" s="90"/>
+      <c r="G16" s="86"/>
+      <c r="H16" s="83"/>
       <c r="I16" s="16"/>
       <c r="M16" s="28"/>
       <c r="N16" s="9"/>
@@ -2328,52 +2328,52 @@
     </row>
     <row r="18" spans="1:25" ht="49.5" hidden="1" customHeight="1">
       <c r="A18" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B18" s="65" t="s">
         <v>14</v>
       </c>
-      <c r="B18" s="65" t="s">
+      <c r="C18" s="66" t="s">
         <v>15</v>
       </c>
-      <c r="C18" s="66" t="s">
+      <c r="D18" s="36" t="s">
         <v>16</v>
       </c>
-      <c r="D18" s="36" t="s">
+      <c r="E18" s="67" t="s">
         <v>17</v>
       </c>
-      <c r="E18" s="67" t="s">
+      <c r="F18" s="36" t="s">
         <v>18</v>
       </c>
-      <c r="F18" s="36" t="s">
+      <c r="G18" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="G18" s="3" t="s">
+      <c r="H18" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="H18" s="4" t="s">
-        <v>21</v>
+      <c r="I18" s="32" t="s">
+        <v>24</v>
       </c>
-      <c r="I18" s="32" t="s">
+      <c r="J18" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="J18" s="32" t="s">
+      <c r="K18" s="32" t="s">
         <v>26</v>
       </c>
-      <c r="K18" s="32" t="s">
+      <c r="L18" s="32" t="s">
         <v>27</v>
       </c>
-      <c r="L18" s="32" t="s">
+      <c r="M18" s="32" t="s">
         <v>28</v>
       </c>
-      <c r="M18" s="32" t="s">
+      <c r="N18" s="32" t="s">
         <v>29</v>
       </c>
-      <c r="N18" s="32" t="s">
+      <c r="O18" s="32" t="s">
         <v>30</v>
       </c>
-      <c r="O18" s="32" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="19" spans="1:25" ht="15.5">
+    </row>
+    <row r="19" spans="1:25" ht="15.6">
       <c r="A19" s="63"/>
       <c r="B19" s="68"/>
       <c r="C19" s="69"/>
@@ -2414,14 +2414,14 @@
       <c r="P20" s="5"/>
     </row>
     <row r="21" spans="1:25" s="37" customFormat="1" ht="15" customHeight="1">
-      <c r="A21" s="98" t="s">
-        <v>52</v>
+      <c r="A21" s="73" t="s">
+        <v>51</v>
       </c>
-      <c r="B21" s="98"/>
-      <c r="C21" s="98"/>
-      <c r="D21" s="98"/>
-      <c r="E21" s="98"/>
-      <c r="F21" s="98"/>
+      <c r="B21" s="73"/>
+      <c r="C21" s="73"/>
+      <c r="D21" s="73"/>
+      <c r="E21" s="73"/>
+      <c r="F21" s="73"/>
       <c r="G21" s="12"/>
       <c r="H21" s="15"/>
       <c r="I21" s="13"/>
@@ -2433,15 +2433,15 @@
       <c r="O21" s="16"/>
       <c r="P21" s="5"/>
     </row>
-    <row r="22" spans="1:25" ht="18.5" thickBot="1">
-      <c r="A22" s="100" t="s">
-        <v>44</v>
+    <row r="22" spans="1:25" ht="18.600000000000001" thickBot="1">
+      <c r="A22" s="76" t="s">
+        <v>43</v>
       </c>
-      <c r="B22" s="101"/>
-      <c r="C22" s="101"/>
-      <c r="D22" s="101"/>
-      <c r="E22" s="101"/>
-      <c r="F22" s="101"/>
+      <c r="B22" s="77"/>
+      <c r="C22" s="77"/>
+      <c r="D22" s="77"/>
+      <c r="E22" s="77"/>
+      <c r="F22" s="77"/>
       <c r="G22" s="53"/>
       <c r="H22" s="53"/>
       <c r="I22" s="53"/>
@@ -2452,44 +2452,44 @@
       <c r="N22" s="54"/>
       <c r="O22" s="54"/>
     </row>
-    <row r="23" spans="1:25" ht="65">
+    <row r="23" spans="1:25" ht="66">
       <c r="A23" s="55" t="s">
+        <v>8</v>
+      </c>
+      <c r="B23" s="39" t="s">
         <v>9</v>
       </c>
-      <c r="B23" s="39" t="s">
+      <c r="C23" s="40" t="s">
+        <v>34</v>
+      </c>
+      <c r="D23" s="40" t="s">
+        <v>35</v>
+      </c>
+      <c r="E23" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="C23" s="40" t="s">
-        <v>35</v>
-      </c>
-      <c r="D23" s="40" t="s">
-        <v>36</v>
-      </c>
-      <c r="E23" s="39" t="s">
+      <c r="F23" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="F23" s="41" t="s">
-        <v>12</v>
+      <c r="G23" s="56"/>
+      <c r="H23" s="79" t="s">
+        <v>57</v>
       </c>
-      <c r="G23" s="56"/>
-      <c r="H23" s="96" t="s">
-        <v>58</v>
-      </c>
-      <c r="I23" s="96"/>
-      <c r="J23" s="96"/>
-      <c r="K23" s="96"/>
-      <c r="L23" s="96"/>
-      <c r="M23" s="96"/>
-      <c r="N23" s="96"/>
-      <c r="O23" s="96"/>
+      <c r="I23" s="79"/>
+      <c r="J23" s="79"/>
+      <c r="K23" s="79"/>
+      <c r="L23" s="79"/>
+      <c r="M23" s="79"/>
+      <c r="N23" s="79"/>
+      <c r="O23" s="79"/>
       <c r="P23" s="8"/>
     </row>
-    <row r="24" spans="1:25" ht="15.5" customHeight="1">
+    <row r="24" spans="1:25" ht="15.45" customHeight="1">
       <c r="A24" s="57" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B24" s="42" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C24" s="43"/>
       <c r="D24" s="44">
@@ -2504,24 +2504,24 @@
         <v>0</v>
       </c>
       <c r="G24" s="56"/>
-      <c r="H24" s="97" t="s">
-        <v>57</v>
+      <c r="H24" s="80" t="s">
+        <v>56</v>
       </c>
-      <c r="I24" s="97"/>
-      <c r="J24" s="97"/>
-      <c r="K24" s="97"/>
-      <c r="L24" s="97"/>
-      <c r="M24" s="97"/>
-      <c r="N24" s="97"/>
-      <c r="O24" s="97"/>
+      <c r="I24" s="80"/>
+      <c r="J24" s="80"/>
+      <c r="K24" s="80"/>
+      <c r="L24" s="80"/>
+      <c r="M24" s="80"/>
+      <c r="N24" s="80"/>
+      <c r="O24" s="80"/>
       <c r="P24" s="5"/>
     </row>
     <row r="25" spans="1:25" ht="18" customHeight="1">
       <c r="A25" s="57" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B25" s="42" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C25" s="43"/>
       <c r="D25" s="44">
@@ -2536,22 +2536,22 @@
         <v>0</v>
       </c>
       <c r="G25" s="56"/>
-      <c r="H25" s="97"/>
-      <c r="I25" s="97"/>
-      <c r="J25" s="97"/>
-      <c r="K25" s="97"/>
-      <c r="L25" s="97"/>
-      <c r="M25" s="97"/>
-      <c r="N25" s="97"/>
-      <c r="O25" s="97"/>
+      <c r="H25" s="80"/>
+      <c r="I25" s="80"/>
+      <c r="J25" s="80"/>
+      <c r="K25" s="80"/>
+      <c r="L25" s="80"/>
+      <c r="M25" s="80"/>
+      <c r="N25" s="80"/>
+      <c r="O25" s="80"/>
       <c r="P25" s="5"/>
     </row>
-    <row r="26" spans="1:25" ht="15.5" customHeight="1">
+    <row r="26" spans="1:25" ht="15.45" customHeight="1">
       <c r="A26" s="57" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B26" s="42" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C26" s="43"/>
       <c r="D26" s="44">
@@ -2566,22 +2566,22 @@
         <v>0</v>
       </c>
       <c r="G26" s="56"/>
-      <c r="H26" s="97"/>
-      <c r="I26" s="97"/>
-      <c r="J26" s="97"/>
-      <c r="K26" s="97"/>
-      <c r="L26" s="97"/>
-      <c r="M26" s="97"/>
-      <c r="N26" s="97"/>
-      <c r="O26" s="97"/>
+      <c r="H26" s="80"/>
+      <c r="I26" s="80"/>
+      <c r="J26" s="80"/>
+      <c r="K26" s="80"/>
+      <c r="L26" s="80"/>
+      <c r="M26" s="80"/>
+      <c r="N26" s="80"/>
+      <c r="O26" s="80"/>
       <c r="P26" s="5"/>
     </row>
-    <row r="27" spans="1:25" ht="15.5" customHeight="1">
+    <row r="27" spans="1:25" ht="15.45" customHeight="1">
       <c r="A27" s="57" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B27" s="42" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C27" s="43"/>
       <c r="D27" s="44">
@@ -2596,22 +2596,22 @@
         <v>0</v>
       </c>
       <c r="G27" s="56"/>
-      <c r="H27" s="97"/>
-      <c r="I27" s="97"/>
-      <c r="J27" s="97"/>
-      <c r="K27" s="97"/>
-      <c r="L27" s="97"/>
-      <c r="M27" s="97"/>
-      <c r="N27" s="97"/>
-      <c r="O27" s="97"/>
+      <c r="H27" s="80"/>
+      <c r="I27" s="80"/>
+      <c r="J27" s="80"/>
+      <c r="K27" s="80"/>
+      <c r="L27" s="80"/>
+      <c r="M27" s="80"/>
+      <c r="N27" s="80"/>
+      <c r="O27" s="80"/>
       <c r="P27" s="5"/>
     </row>
-    <row r="28" spans="1:25" ht="15.5" customHeight="1">
+    <row r="28" spans="1:25" ht="15.45" customHeight="1">
       <c r="A28" s="57" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B28" s="42" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C28" s="47"/>
       <c r="D28" s="44">
@@ -2626,22 +2626,22 @@
         <v>0</v>
       </c>
       <c r="G28" s="56"/>
-      <c r="H28" s="97"/>
-      <c r="I28" s="97"/>
-      <c r="J28" s="97"/>
-      <c r="K28" s="97"/>
-      <c r="L28" s="97"/>
-      <c r="M28" s="97"/>
-      <c r="N28" s="97"/>
-      <c r="O28" s="97"/>
+      <c r="H28" s="80"/>
+      <c r="I28" s="80"/>
+      <c r="J28" s="80"/>
+      <c r="K28" s="80"/>
+      <c r="L28" s="80"/>
+      <c r="M28" s="80"/>
+      <c r="N28" s="80"/>
+      <c r="O28" s="80"/>
       <c r="P28" s="5"/>
     </row>
     <row r="29" spans="1:25" ht="15" customHeight="1">
       <c r="A29" s="58" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B29" s="42" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C29" s="47"/>
       <c r="D29" s="44">
@@ -2668,10 +2668,10 @@
     </row>
     <row r="30" spans="1:25" ht="15" customHeight="1">
       <c r="A30" s="58" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B30" s="42" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C30" s="47"/>
       <c r="D30" s="44">
@@ -2708,7 +2708,7 @@
     <row r="31" spans="1:25" ht="15.75" customHeight="1" thickBot="1">
       <c r="A31" s="60"/>
       <c r="B31" s="48" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C31" s="49"/>
       <c r="D31" s="50"/>
@@ -2765,23 +2765,23 @@
       <c r="Y32" s="5"/>
     </row>
     <row r="33" spans="1:25" ht="18">
-      <c r="A33" s="99" t="s">
-        <v>56</v>
+      <c r="A33" s="74" t="s">
+        <v>55</v>
       </c>
-      <c r="B33" s="99"/>
-      <c r="C33" s="99"/>
-      <c r="D33" s="99"/>
-      <c r="E33" s="99"/>
-      <c r="F33" s="99"/>
-      <c r="G33" s="99"/>
-      <c r="H33" s="99"/>
-      <c r="I33" s="99"/>
-      <c r="J33" s="99"/>
-      <c r="K33" s="99"/>
-      <c r="L33" s="99"/>
-      <c r="M33" s="99"/>
-      <c r="N33" s="99"/>
-      <c r="O33" s="99"/>
+      <c r="B33" s="74"/>
+      <c r="C33" s="74"/>
+      <c r="D33" s="74"/>
+      <c r="E33" s="74"/>
+      <c r="F33" s="74"/>
+      <c r="G33" s="74"/>
+      <c r="H33" s="74"/>
+      <c r="I33" s="74"/>
+      <c r="J33" s="74"/>
+      <c r="K33" s="74"/>
+      <c r="L33" s="74"/>
+      <c r="M33" s="74"/>
+      <c r="N33" s="74"/>
+      <c r="O33" s="74"/>
       <c r="P33" s="17"/>
       <c r="Q33" s="5"/>
       <c r="R33" s="5"/>
@@ -2795,17 +2795,17 @@
     </row>
     <row r="34" spans="1:25" ht="18" customHeight="1">
       <c r="A34" s="75" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B34" s="75"/>
       <c r="C34" s="75"/>
       <c r="D34" s="75"/>
       <c r="E34" s="75"/>
       <c r="F34" s="61" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G34" s="19" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H34" s="19"/>
       <c r="I34" s="19"/>
@@ -2826,7 +2826,7 @@
       <c r="X34" s="5"/>
       <c r="Y34" s="5"/>
     </row>
-    <row r="35" spans="1:25" ht="15.5" customHeight="1">
+    <row r="35" spans="1:25" ht="15.45" customHeight="1">
       <c r="A35" s="17"/>
       <c r="B35" s="17"/>
       <c r="C35" s="17"/>
@@ -2855,11 +2855,11 @@
     </row>
     <row r="36" spans="1:25" ht="18" customHeight="1">
       <c r="A36" s="75" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B36" s="75"/>
       <c r="C36" s="75" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D36" s="75"/>
       <c r="E36" s="75"/>
@@ -2868,7 +2868,7 @@
       <c r="H36" s="17"/>
       <c r="I36" s="23"/>
       <c r="L36" s="75" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="M36" s="75"/>
       <c r="N36" s="75"/>
@@ -2880,11 +2880,11 @@
     </row>
     <row r="37" spans="1:25" ht="18" customHeight="1">
       <c r="A37" s="75" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B37" s="75"/>
       <c r="C37" s="75" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D37" s="75"/>
       <c r="E37" s="75"/>
@@ -2893,7 +2893,7 @@
       <c r="H37" s="17"/>
       <c r="I37" s="23"/>
       <c r="L37" s="75" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="M37" s="75"/>
       <c r="N37" s="75"/>
@@ -2906,21 +2906,21 @@
     <row r="38" spans="1:25" ht="18" customHeight="1">
       <c r="A38" s="8"/>
       <c r="B38" s="20"/>
-      <c r="C38" s="95" t="s">
-        <v>66</v>
+      <c r="C38" s="78" t="s">
+        <v>65</v>
       </c>
-      <c r="D38" s="95"/>
-      <c r="E38" s="95"/>
+      <c r="D38" s="78"/>
+      <c r="E38" s="78"/>
       <c r="F38" s="23"/>
       <c r="G38" s="23"/>
       <c r="H38" s="23"/>
       <c r="I38" s="23"/>
-      <c r="L38" s="95" t="s">
-        <v>70</v>
+      <c r="L38" s="78" t="s">
+        <v>69</v>
       </c>
-      <c r="M38" s="95"/>
-      <c r="N38" s="95"/>
-      <c r="O38" s="95"/>
+      <c r="M38" s="78"/>
+      <c r="N38" s="78"/>
+      <c r="O38" s="78"/>
       <c r="P38" s="8"/>
       <c r="Q38" s="8"/>
       <c r="R38" s="8"/>
@@ -2929,21 +2929,21 @@
     <row r="39" spans="1:25" ht="18" customHeight="1">
       <c r="A39" s="8"/>
       <c r="B39" s="20"/>
-      <c r="C39" s="95" t="s">
-        <v>67</v>
+      <c r="C39" s="78" t="s">
+        <v>66</v>
       </c>
-      <c r="D39" s="95"/>
-      <c r="E39" s="95"/>
+      <c r="D39" s="78"/>
+      <c r="E39" s="78"/>
       <c r="F39" s="23"/>
       <c r="G39" s="23"/>
       <c r="H39" s="23"/>
       <c r="I39" s="23"/>
-      <c r="L39" s="95" t="s">
-        <v>71</v>
+      <c r="L39" s="78" t="s">
+        <v>70</v>
       </c>
-      <c r="M39" s="95"/>
-      <c r="N39" s="95"/>
-      <c r="O39" s="95"/>
+      <c r="M39" s="78"/>
+      <c r="N39" s="78"/>
+      <c r="O39" s="78"/>
       <c r="P39" s="21"/>
       <c r="Q39" s="21"/>
       <c r="R39" s="21"/>
@@ -3651,7 +3651,7 @@
       <c r="X65" s="5"/>
       <c r="Y65" s="5"/>
     </row>
-    <row r="66" spans="1:25" ht="59" customHeight="1">
+    <row r="66" spans="1:25" ht="58.95" customHeight="1">
       <c r="A66" s="5"/>
       <c r="B66" s="5"/>
       <c r="C66" s="5"/>
@@ -4056,7 +4056,7 @@
       <c r="X80" s="5"/>
       <c r="Y80" s="5"/>
     </row>
-    <row r="81" spans="1:25" ht="46" customHeight="1">
+    <row r="81" spans="1:25" ht="46.05" customHeight="1">
       <c r="A81" s="5"/>
       <c r="B81" s="5"/>
       <c r="C81" s="5"/>
@@ -27810,27 +27810,6 @@
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
   <mergeCells count="37">
-    <mergeCell ref="A21:F21"/>
-    <mergeCell ref="A33:O33"/>
-    <mergeCell ref="A34:E34"/>
-    <mergeCell ref="A36:B36"/>
-    <mergeCell ref="A37:B37"/>
-    <mergeCell ref="A22:F22"/>
-    <mergeCell ref="C38:E38"/>
-    <mergeCell ref="C36:E36"/>
-    <mergeCell ref="H23:O23"/>
-    <mergeCell ref="H24:O28"/>
-    <mergeCell ref="C39:E39"/>
-    <mergeCell ref="C37:E37"/>
-    <mergeCell ref="L38:O38"/>
-    <mergeCell ref="L39:O39"/>
-    <mergeCell ref="K8:M8"/>
-    <mergeCell ref="H15:H16"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="D15:D16"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="F15:F16"/>
     <mergeCell ref="N8:O8"/>
     <mergeCell ref="K9:O9"/>
     <mergeCell ref="L36:O36"/>
@@ -27847,6 +27826,27 @@
     <mergeCell ref="A11:O11"/>
     <mergeCell ref="A12:O12"/>
     <mergeCell ref="A14:O14"/>
+    <mergeCell ref="K8:M8"/>
+    <mergeCell ref="H15:H16"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="D15:D16"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="F15:F16"/>
+    <mergeCell ref="C38:E38"/>
+    <mergeCell ref="C36:E36"/>
+    <mergeCell ref="H23:O23"/>
+    <mergeCell ref="H24:O28"/>
+    <mergeCell ref="C39:E39"/>
+    <mergeCell ref="C37:E37"/>
+    <mergeCell ref="L38:O38"/>
+    <mergeCell ref="L39:O39"/>
+    <mergeCell ref="A21:F21"/>
+    <mergeCell ref="A33:O33"/>
+    <mergeCell ref="A34:E34"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="A22:F22"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>

</xml_diff>

<commit_message>
change the structure, fix a lot of stuff, add a new report (#42)
* change the structure, fix a lot of stuff, add a new report

* fix certificates password issue

* fix certificate
</commit_message>
<xml_diff>
--- a/Mil.Paperwork.Domain/Templates/ResidualValueReportTemplate.xlsx
+++ b/Mil.Paperwork.Domain/Templates/ResidualValueReportTemplate.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\Projects\Mil.Paperwork.WriteOff\Mil.Paperwork.Domain\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45E1B699-A6AB-4C5E-B963-C8CF80867B06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7E80A4F-BCC2-4309-9075-5A94E82FA98C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Відомість" sheetId="1" r:id="rId1"/>
@@ -68,9 +68,6 @@
   </si>
   <si>
     <t>ЗАТВЕРДЖУЮ</t>
-  </si>
-  <si>
-    <t>"____" __________ 2025 року</t>
   </si>
   <si>
     <t>ВІДОМІСТЬ</t>
@@ -303,6 +300,9 @@
   </si>
   <si>
     <t>Командир військової частини [MIL_UNIT]</t>
+  </si>
+  <si>
+    <t>"____" __________ 2026 року</t>
   </si>
 </sst>
 </file>
@@ -1119,13 +1119,62 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1149,57 +1198,8 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1924,24 +1924,24 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:Y1003"/>
-  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="8.54296875" style="6" customWidth="1"/>
-    <col min="2" max="2" width="40.1796875" style="6" customWidth="1"/>
-    <col min="3" max="3" width="8.6328125" style="6" customWidth="1"/>
-    <col min="4" max="4" width="9.81640625" style="6" customWidth="1"/>
-    <col min="5" max="5" width="24.36328125" style="6" customWidth="1"/>
-    <col min="6" max="6" width="13.36328125" style="6" customWidth="1"/>
-    <col min="7" max="7" width="12.26953125" style="6" customWidth="1"/>
-    <col min="8" max="8" width="18.81640625" style="6" customWidth="1"/>
-    <col min="9" max="11" width="7.7265625" style="6" customWidth="1"/>
-    <col min="12" max="13" width="14.453125" style="6" customWidth="1"/>
-    <col min="14" max="14" width="14.54296875" style="6" customWidth="1"/>
-    <col min="15" max="15" width="14.453125" style="6" customWidth="1"/>
-    <col min="16" max="25" width="13.26953125" style="6" customWidth="1"/>
-    <col min="26" max="998" width="14.453125" style="6"/>
-    <col min="999" max="9998" width="15.1796875" style="6" customWidth="1"/>
-    <col min="9999" max="16384" width="16.1796875" style="6" customWidth="1"/>
+    <col min="1" max="1" width="8.5546875" style="6" customWidth="1"/>
+    <col min="2" max="2" width="40.21875" style="6" customWidth="1"/>
+    <col min="3" max="3" width="8.6640625" style="6" customWidth="1"/>
+    <col min="4" max="4" width="9.77734375" style="6" customWidth="1"/>
+    <col min="5" max="5" width="24.33203125" style="6" customWidth="1"/>
+    <col min="6" max="6" width="13.33203125" style="6" customWidth="1"/>
+    <col min="7" max="7" width="12.21875" style="6" customWidth="1"/>
+    <col min="8" max="8" width="18.77734375" style="6" customWidth="1"/>
+    <col min="9" max="11" width="7.77734375" style="6" customWidth="1"/>
+    <col min="12" max="13" width="14.44140625" style="6" customWidth="1"/>
+    <col min="14" max="14" width="14.5546875" style="6" customWidth="1"/>
+    <col min="15" max="15" width="14.44140625" style="6" customWidth="1"/>
+    <col min="16" max="25" width="13.21875" style="6" customWidth="1"/>
+    <col min="26" max="998" width="14.44140625" style="6"/>
+    <col min="999" max="9998" width="15.21875" style="6" customWidth="1"/>
+    <col min="9999" max="16384" width="16.21875" style="6" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="12.75" customHeight="1">
@@ -1999,10 +1999,10 @@
       <c r="Y2" s="5"/>
     </row>
     <row r="3" spans="1:25" ht="12.75" customHeight="1">
-      <c r="A3" s="76" t="s">
-        <v>63</v>
+      <c r="A3" s="93" t="s">
+        <v>62</v>
       </c>
-      <c r="B3" s="77"/>
+      <c r="B3" s="94"/>
       <c r="C3" s="5"/>
       <c r="D3" s="5"/>
       <c r="E3" s="5"/>
@@ -2028,14 +2028,14 @@
       <c r="Y3" s="5"/>
     </row>
     <row r="4" spans="1:25" ht="12.75" customHeight="1">
-      <c r="A4" s="78" t="s">
+      <c r="A4" s="95" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="77"/>
-      <c r="C4" s="80" t="s">
-        <v>24</v>
+      <c r="B4" s="94"/>
+      <c r="C4" s="97" t="s">
+        <v>23</v>
       </c>
-      <c r="D4" s="81"/>
+      <c r="D4" s="98"/>
       <c r="E4" s="27"/>
       <c r="F4" s="5"/>
       <c r="G4" s="5"/>
@@ -2086,19 +2086,19 @@
       <c r="Y5" s="5"/>
     </row>
     <row r="6" spans="1:25" ht="18" customHeight="1">
-      <c r="A6" s="79"/>
-      <c r="B6" s="77"/>
+      <c r="A6" s="96"/>
+      <c r="B6" s="94"/>
       <c r="C6" s="7"/>
       <c r="D6" s="7"/>
       <c r="E6" s="7"/>
       <c r="F6" s="7"/>
-      <c r="K6" s="74" t="s">
+      <c r="K6" s="92" t="s">
         <v>1</v>
       </c>
-      <c r="L6" s="74"/>
-      <c r="M6" s="74"/>
-      <c r="N6" s="74"/>
-      <c r="O6" s="74"/>
+      <c r="L6" s="92"/>
+      <c r="M6" s="92"/>
+      <c r="N6" s="92"/>
+      <c r="O6" s="92"/>
       <c r="P6" s="20"/>
     </row>
     <row r="7" spans="1:25" ht="18">
@@ -2108,12 +2108,12 @@
       <c r="D7" s="7"/>
       <c r="E7" s="7"/>
       <c r="K7" s="75" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
-      <c r="L7" s="74"/>
-      <c r="M7" s="74"/>
-      <c r="N7" s="74"/>
-      <c r="O7" s="74"/>
+      <c r="L7" s="92"/>
+      <c r="M7" s="92"/>
+      <c r="N7" s="92"/>
+      <c r="O7" s="92"/>
       <c r="P7" s="20"/>
     </row>
     <row r="8" spans="1:25" ht="18" customHeight="1">
@@ -2122,15 +2122,15 @@
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
       <c r="E8" s="7"/>
-      <c r="K8" s="87" t="s">
+      <c r="K8" s="81" t="s">
+        <v>60</v>
+      </c>
+      <c r="L8" s="81"/>
+      <c r="M8" s="81"/>
+      <c r="N8" s="91" t="s">
         <v>61</v>
       </c>
-      <c r="L8" s="87"/>
-      <c r="M8" s="87"/>
-      <c r="N8" s="73" t="s">
-        <v>62</v>
-      </c>
-      <c r="O8" s="73"/>
+      <c r="O8" s="91"/>
       <c r="P8" s="8"/>
     </row>
     <row r="9" spans="1:25" ht="24.75" customHeight="1">
@@ -2139,13 +2139,13 @@
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
       <c r="E9" s="7"/>
-      <c r="K9" s="74" t="s">
-        <v>2</v>
+      <c r="K9" s="92" t="s">
+        <v>72</v>
       </c>
-      <c r="L9" s="74"/>
-      <c r="M9" s="74"/>
-      <c r="N9" s="74"/>
-      <c r="O9" s="74"/>
+      <c r="L9" s="92"/>
+      <c r="M9" s="92"/>
+      <c r="N9" s="92"/>
+      <c r="O9" s="92"/>
       <c r="P9" s="20"/>
     </row>
     <row r="10" spans="1:25" ht="18" customHeight="1">
@@ -2166,23 +2166,23 @@
       <c r="Y10" s="8"/>
     </row>
     <row r="11" spans="1:25" ht="18" customHeight="1">
-      <c r="A11" s="86" t="s">
-        <v>3</v>
+      <c r="A11" s="101" t="s">
+        <v>2</v>
       </c>
-      <c r="B11" s="86"/>
-      <c r="C11" s="86"/>
-      <c r="D11" s="86"/>
-      <c r="E11" s="86"/>
-      <c r="F11" s="86"/>
-      <c r="G11" s="86"/>
-      <c r="H11" s="86"/>
-      <c r="I11" s="86"/>
-      <c r="J11" s="86"/>
-      <c r="K11" s="86"/>
-      <c r="L11" s="86"/>
-      <c r="M11" s="86"/>
-      <c r="N11" s="86"/>
-      <c r="O11" s="86"/>
+      <c r="B11" s="101"/>
+      <c r="C11" s="101"/>
+      <c r="D11" s="101"/>
+      <c r="E11" s="101"/>
+      <c r="F11" s="101"/>
+      <c r="G11" s="101"/>
+      <c r="H11" s="101"/>
+      <c r="I11" s="101"/>
+      <c r="J11" s="101"/>
+      <c r="K11" s="101"/>
+      <c r="L11" s="101"/>
+      <c r="M11" s="101"/>
+      <c r="N11" s="101"/>
+      <c r="O11" s="101"/>
       <c r="P11" s="8"/>
       <c r="Q11" s="8"/>
       <c r="R11" s="8"/>
@@ -2195,87 +2195,87 @@
       <c r="Y11" s="8"/>
     </row>
     <row r="12" spans="1:25" ht="18" customHeight="1">
-      <c r="A12" s="83" t="s">
+      <c r="A12" s="100" t="s">
+        <v>32</v>
+      </c>
+      <c r="B12" s="100"/>
+      <c r="C12" s="100"/>
+      <c r="D12" s="100"/>
+      <c r="E12" s="100"/>
+      <c r="F12" s="100"/>
+      <c r="G12" s="100"/>
+      <c r="H12" s="100"/>
+      <c r="I12" s="100"/>
+      <c r="J12" s="100"/>
+      <c r="K12" s="100"/>
+      <c r="L12" s="100"/>
+      <c r="M12" s="100"/>
+      <c r="N12" s="100"/>
+      <c r="O12" s="100"/>
+      <c r="P12" s="8"/>
+    </row>
+    <row r="13" spans="1:25" s="37" customFormat="1" ht="18" customHeight="1">
+      <c r="A13" s="100" t="s">
+        <v>58</v>
+      </c>
+      <c r="B13" s="100"/>
+      <c r="C13" s="100"/>
+      <c r="D13" s="100"/>
+      <c r="E13" s="100"/>
+      <c r="F13" s="100"/>
+      <c r="G13" s="100"/>
+      <c r="H13" s="100"/>
+      <c r="I13" s="100"/>
+      <c r="J13" s="100"/>
+      <c r="K13" s="100"/>
+      <c r="L13" s="100"/>
+      <c r="M13" s="100"/>
+      <c r="N13" s="100"/>
+      <c r="O13" s="100"/>
+      <c r="P13" s="8"/>
+    </row>
+    <row r="14" spans="1:25" ht="18" customHeight="1">
+      <c r="A14" s="101"/>
+      <c r="B14" s="101"/>
+      <c r="C14" s="101"/>
+      <c r="D14" s="101"/>
+      <c r="E14" s="101"/>
+      <c r="F14" s="101"/>
+      <c r="G14" s="101"/>
+      <c r="H14" s="101"/>
+      <c r="I14" s="101"/>
+      <c r="J14" s="101"/>
+      <c r="K14" s="101"/>
+      <c r="L14" s="101"/>
+      <c r="M14" s="101"/>
+      <c r="N14" s="101"/>
+      <c r="O14" s="101"/>
+      <c r="P14" s="8"/>
+    </row>
+    <row r="15" spans="1:25" ht="67.95" customHeight="1">
+      <c r="A15" s="84" t="s">
+        <v>3</v>
+      </c>
+      <c r="B15" s="84" t="s">
+        <v>4</v>
+      </c>
+      <c r="C15" s="84" t="s">
+        <v>5</v>
+      </c>
+      <c r="D15" s="87" t="s">
+        <v>6</v>
+      </c>
+      <c r="E15" s="99" t="s">
         <v>33</v>
       </c>
-      <c r="B12" s="83"/>
-      <c r="C12" s="83"/>
-      <c r="D12" s="83"/>
-      <c r="E12" s="83"/>
-      <c r="F12" s="83"/>
-      <c r="G12" s="83"/>
-      <c r="H12" s="83"/>
-      <c r="I12" s="83"/>
-      <c r="J12" s="83"/>
-      <c r="K12" s="83"/>
-      <c r="L12" s="83"/>
-      <c r="M12" s="83"/>
-      <c r="N12" s="83"/>
-      <c r="O12" s="83"/>
-      <c r="P12" s="8"/>
-    </row>
-    <row r="13" spans="1:25" s="37" customFormat="1" ht="18" customHeight="1">
-      <c r="A13" s="83" t="s">
+      <c r="F15" s="89" t="s">
+        <v>21</v>
+      </c>
+      <c r="G15" s="84" t="s">
         <v>59</v>
       </c>
-      <c r="B13" s="83"/>
-      <c r="C13" s="83"/>
-      <c r="D13" s="83"/>
-      <c r="E13" s="83"/>
-      <c r="F13" s="83"/>
-      <c r="G13" s="83"/>
-      <c r="H13" s="83"/>
-      <c r="I13" s="83"/>
-      <c r="J13" s="83"/>
-      <c r="K13" s="83"/>
-      <c r="L13" s="83"/>
-      <c r="M13" s="83"/>
-      <c r="N13" s="83"/>
-      <c r="O13" s="83"/>
-      <c r="P13" s="8"/>
-    </row>
-    <row r="14" spans="1:25" ht="18" customHeight="1">
-      <c r="A14" s="86"/>
-      <c r="B14" s="86"/>
-      <c r="C14" s="86"/>
-      <c r="D14" s="86"/>
-      <c r="E14" s="86"/>
-      <c r="F14" s="86"/>
-      <c r="G14" s="86"/>
-      <c r="H14" s="86"/>
-      <c r="I14" s="86"/>
-      <c r="J14" s="86"/>
-      <c r="K14" s="86"/>
-      <c r="L14" s="86"/>
-      <c r="M14" s="86"/>
-      <c r="N14" s="86"/>
-      <c r="O14" s="86"/>
-      <c r="P14" s="8"/>
-    </row>
-    <row r="15" spans="1:25" ht="68" customHeight="1">
-      <c r="A15" s="84" t="s">
-        <v>4</v>
-      </c>
-      <c r="B15" s="84" t="s">
-        <v>5</v>
-      </c>
-      <c r="C15" s="84" t="s">
-        <v>6</v>
-      </c>
-      <c r="D15" s="91" t="s">
+      <c r="H15" s="82" t="s">
         <v>7</v>
-      </c>
-      <c r="E15" s="82" t="s">
-        <v>34</v>
-      </c>
-      <c r="F15" s="93" t="s">
-        <v>22</v>
-      </c>
-      <c r="G15" s="84" t="s">
-        <v>60</v>
-      </c>
-      <c r="H15" s="88" t="s">
-        <v>8</v>
       </c>
       <c r="I15" s="28"/>
       <c r="M15" s="28"/>
@@ -2283,14 +2283,14 @@
       <c r="O15" s="10"/>
     </row>
     <row r="16" spans="1:25" ht="24" customHeight="1">
-      <c r="A16" s="90"/>
-      <c r="B16" s="85"/>
-      <c r="C16" s="85"/>
-      <c r="D16" s="92"/>
-      <c r="E16" s="82"/>
-      <c r="F16" s="94"/>
-      <c r="G16" s="85"/>
-      <c r="H16" s="89"/>
+      <c r="A16" s="85"/>
+      <c r="B16" s="86"/>
+      <c r="C16" s="86"/>
+      <c r="D16" s="88"/>
+      <c r="E16" s="99"/>
+      <c r="F16" s="90"/>
+      <c r="G16" s="86"/>
+      <c r="H16" s="83"/>
       <c r="I16" s="16"/>
       <c r="M16" s="28"/>
       <c r="N16" s="9"/>
@@ -2328,52 +2328,52 @@
     </row>
     <row r="18" spans="1:25" ht="49.5" hidden="1" customHeight="1">
       <c r="A18" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B18" s="65" t="s">
         <v>14</v>
       </c>
-      <c r="B18" s="65" t="s">
+      <c r="C18" s="66" t="s">
         <v>15</v>
       </c>
-      <c r="C18" s="66" t="s">
+      <c r="D18" s="36" t="s">
         <v>16</v>
       </c>
-      <c r="D18" s="36" t="s">
+      <c r="E18" s="67" t="s">
         <v>17</v>
       </c>
-      <c r="E18" s="67" t="s">
+      <c r="F18" s="36" t="s">
         <v>18</v>
       </c>
-      <c r="F18" s="36" t="s">
+      <c r="G18" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="G18" s="3" t="s">
+      <c r="H18" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="H18" s="4" t="s">
-        <v>21</v>
+      <c r="I18" s="32" t="s">
+        <v>24</v>
       </c>
-      <c r="I18" s="32" t="s">
+      <c r="J18" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="J18" s="32" t="s">
+      <c r="K18" s="32" t="s">
         <v>26</v>
       </c>
-      <c r="K18" s="32" t="s">
+      <c r="L18" s="32" t="s">
         <v>27</v>
       </c>
-      <c r="L18" s="32" t="s">
+      <c r="M18" s="32" t="s">
         <v>28</v>
       </c>
-      <c r="M18" s="32" t="s">
+      <c r="N18" s="32" t="s">
         <v>29</v>
       </c>
-      <c r="N18" s="32" t="s">
+      <c r="O18" s="32" t="s">
         <v>30</v>
       </c>
-      <c r="O18" s="32" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="19" spans="1:25" ht="15.5">
+    </row>
+    <row r="19" spans="1:25" ht="15.6">
       <c r="A19" s="63"/>
       <c r="B19" s="68"/>
       <c r="C19" s="69"/>
@@ -2414,14 +2414,14 @@
       <c r="P20" s="5"/>
     </row>
     <row r="21" spans="1:25" s="37" customFormat="1" ht="15" customHeight="1">
-      <c r="A21" s="98" t="s">
-        <v>52</v>
+      <c r="A21" s="73" t="s">
+        <v>51</v>
       </c>
-      <c r="B21" s="98"/>
-      <c r="C21" s="98"/>
-      <c r="D21" s="98"/>
-      <c r="E21" s="98"/>
-      <c r="F21" s="98"/>
+      <c r="B21" s="73"/>
+      <c r="C21" s="73"/>
+      <c r="D21" s="73"/>
+      <c r="E21" s="73"/>
+      <c r="F21" s="73"/>
       <c r="G21" s="12"/>
       <c r="H21" s="15"/>
       <c r="I21" s="13"/>
@@ -2433,15 +2433,15 @@
       <c r="O21" s="16"/>
       <c r="P21" s="5"/>
     </row>
-    <row r="22" spans="1:25" ht="18.5" thickBot="1">
-      <c r="A22" s="100" t="s">
-        <v>44</v>
+    <row r="22" spans="1:25" ht="18.600000000000001" thickBot="1">
+      <c r="A22" s="76" t="s">
+        <v>43</v>
       </c>
-      <c r="B22" s="101"/>
-      <c r="C22" s="101"/>
-      <c r="D22" s="101"/>
-      <c r="E22" s="101"/>
-      <c r="F22" s="101"/>
+      <c r="B22" s="77"/>
+      <c r="C22" s="77"/>
+      <c r="D22" s="77"/>
+      <c r="E22" s="77"/>
+      <c r="F22" s="77"/>
       <c r="G22" s="53"/>
       <c r="H22" s="53"/>
       <c r="I22" s="53"/>
@@ -2452,44 +2452,44 @@
       <c r="N22" s="54"/>
       <c r="O22" s="54"/>
     </row>
-    <row r="23" spans="1:25" ht="65">
+    <row r="23" spans="1:25" ht="66">
       <c r="A23" s="55" t="s">
+        <v>8</v>
+      </c>
+      <c r="B23" s="39" t="s">
         <v>9</v>
       </c>
-      <c r="B23" s="39" t="s">
+      <c r="C23" s="40" t="s">
+        <v>34</v>
+      </c>
+      <c r="D23" s="40" t="s">
+        <v>35</v>
+      </c>
+      <c r="E23" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="C23" s="40" t="s">
-        <v>35</v>
-      </c>
-      <c r="D23" s="40" t="s">
-        <v>36</v>
-      </c>
-      <c r="E23" s="39" t="s">
+      <c r="F23" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="F23" s="41" t="s">
-        <v>12</v>
+      <c r="G23" s="56"/>
+      <c r="H23" s="79" t="s">
+        <v>57</v>
       </c>
-      <c r="G23" s="56"/>
-      <c r="H23" s="96" t="s">
-        <v>58</v>
-      </c>
-      <c r="I23" s="96"/>
-      <c r="J23" s="96"/>
-      <c r="K23" s="96"/>
-      <c r="L23" s="96"/>
-      <c r="M23" s="96"/>
-      <c r="N23" s="96"/>
-      <c r="O23" s="96"/>
+      <c r="I23" s="79"/>
+      <c r="J23" s="79"/>
+      <c r="K23" s="79"/>
+      <c r="L23" s="79"/>
+      <c r="M23" s="79"/>
+      <c r="N23" s="79"/>
+      <c r="O23" s="79"/>
       <c r="P23" s="8"/>
     </row>
-    <row r="24" spans="1:25" ht="15.5" customHeight="1">
+    <row r="24" spans="1:25" ht="15.45" customHeight="1">
       <c r="A24" s="57" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B24" s="42" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C24" s="43"/>
       <c r="D24" s="44">
@@ -2504,24 +2504,24 @@
         <v>0</v>
       </c>
       <c r="G24" s="56"/>
-      <c r="H24" s="97" t="s">
-        <v>57</v>
+      <c r="H24" s="80" t="s">
+        <v>56</v>
       </c>
-      <c r="I24" s="97"/>
-      <c r="J24" s="97"/>
-      <c r="K24" s="97"/>
-      <c r="L24" s="97"/>
-      <c r="M24" s="97"/>
-      <c r="N24" s="97"/>
-      <c r="O24" s="97"/>
+      <c r="I24" s="80"/>
+      <c r="J24" s="80"/>
+      <c r="K24" s="80"/>
+      <c r="L24" s="80"/>
+      <c r="M24" s="80"/>
+      <c r="N24" s="80"/>
+      <c r="O24" s="80"/>
       <c r="P24" s="5"/>
     </row>
     <row r="25" spans="1:25" ht="18" customHeight="1">
       <c r="A25" s="57" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B25" s="42" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C25" s="43"/>
       <c r="D25" s="44">
@@ -2536,22 +2536,22 @@
         <v>0</v>
       </c>
       <c r="G25" s="56"/>
-      <c r="H25" s="97"/>
-      <c r="I25" s="97"/>
-      <c r="J25" s="97"/>
-      <c r="K25" s="97"/>
-      <c r="L25" s="97"/>
-      <c r="M25" s="97"/>
-      <c r="N25" s="97"/>
-      <c r="O25" s="97"/>
+      <c r="H25" s="80"/>
+      <c r="I25" s="80"/>
+      <c r="J25" s="80"/>
+      <c r="K25" s="80"/>
+      <c r="L25" s="80"/>
+      <c r="M25" s="80"/>
+      <c r="N25" s="80"/>
+      <c r="O25" s="80"/>
       <c r="P25" s="5"/>
     </row>
-    <row r="26" spans="1:25" ht="15.5" customHeight="1">
+    <row r="26" spans="1:25" ht="15.45" customHeight="1">
       <c r="A26" s="57" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B26" s="42" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C26" s="43"/>
       <c r="D26" s="44">
@@ -2566,22 +2566,22 @@
         <v>0</v>
       </c>
       <c r="G26" s="56"/>
-      <c r="H26" s="97"/>
-      <c r="I26" s="97"/>
-      <c r="J26" s="97"/>
-      <c r="K26" s="97"/>
-      <c r="L26" s="97"/>
-      <c r="M26" s="97"/>
-      <c r="N26" s="97"/>
-      <c r="O26" s="97"/>
+      <c r="H26" s="80"/>
+      <c r="I26" s="80"/>
+      <c r="J26" s="80"/>
+      <c r="K26" s="80"/>
+      <c r="L26" s="80"/>
+      <c r="M26" s="80"/>
+      <c r="N26" s="80"/>
+      <c r="O26" s="80"/>
       <c r="P26" s="5"/>
     </row>
-    <row r="27" spans="1:25" ht="15.5" customHeight="1">
+    <row r="27" spans="1:25" ht="15.45" customHeight="1">
       <c r="A27" s="57" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B27" s="42" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C27" s="43"/>
       <c r="D27" s="44">
@@ -2596,22 +2596,22 @@
         <v>0</v>
       </c>
       <c r="G27" s="56"/>
-      <c r="H27" s="97"/>
-      <c r="I27" s="97"/>
-      <c r="J27" s="97"/>
-      <c r="K27" s="97"/>
-      <c r="L27" s="97"/>
-      <c r="M27" s="97"/>
-      <c r="N27" s="97"/>
-      <c r="O27" s="97"/>
+      <c r="H27" s="80"/>
+      <c r="I27" s="80"/>
+      <c r="J27" s="80"/>
+      <c r="K27" s="80"/>
+      <c r="L27" s="80"/>
+      <c r="M27" s="80"/>
+      <c r="N27" s="80"/>
+      <c r="O27" s="80"/>
       <c r="P27" s="5"/>
     </row>
-    <row r="28" spans="1:25" ht="15.5" customHeight="1">
+    <row r="28" spans="1:25" ht="15.45" customHeight="1">
       <c r="A28" s="57" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B28" s="42" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C28" s="47"/>
       <c r="D28" s="44">
@@ -2626,22 +2626,22 @@
         <v>0</v>
       </c>
       <c r="G28" s="56"/>
-      <c r="H28" s="97"/>
-      <c r="I28" s="97"/>
-      <c r="J28" s="97"/>
-      <c r="K28" s="97"/>
-      <c r="L28" s="97"/>
-      <c r="M28" s="97"/>
-      <c r="N28" s="97"/>
-      <c r="O28" s="97"/>
+      <c r="H28" s="80"/>
+      <c r="I28" s="80"/>
+      <c r="J28" s="80"/>
+      <c r="K28" s="80"/>
+      <c r="L28" s="80"/>
+      <c r="M28" s="80"/>
+      <c r="N28" s="80"/>
+      <c r="O28" s="80"/>
       <c r="P28" s="5"/>
     </row>
     <row r="29" spans="1:25" ht="15" customHeight="1">
       <c r="A29" s="58" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B29" s="42" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C29" s="47"/>
       <c r="D29" s="44">
@@ -2668,10 +2668,10 @@
     </row>
     <row r="30" spans="1:25" ht="15" customHeight="1">
       <c r="A30" s="58" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B30" s="42" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C30" s="47"/>
       <c r="D30" s="44">
@@ -2708,7 +2708,7 @@
     <row r="31" spans="1:25" ht="15.75" customHeight="1" thickBot="1">
       <c r="A31" s="60"/>
       <c r="B31" s="48" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C31" s="49"/>
       <c r="D31" s="50"/>
@@ -2765,23 +2765,23 @@
       <c r="Y32" s="5"/>
     </row>
     <row r="33" spans="1:25" ht="18">
-      <c r="A33" s="99" t="s">
-        <v>56</v>
+      <c r="A33" s="74" t="s">
+        <v>55</v>
       </c>
-      <c r="B33" s="99"/>
-      <c r="C33" s="99"/>
-      <c r="D33" s="99"/>
-      <c r="E33" s="99"/>
-      <c r="F33" s="99"/>
-      <c r="G33" s="99"/>
-      <c r="H33" s="99"/>
-      <c r="I33" s="99"/>
-      <c r="J33" s="99"/>
-      <c r="K33" s="99"/>
-      <c r="L33" s="99"/>
-      <c r="M33" s="99"/>
-      <c r="N33" s="99"/>
-      <c r="O33" s="99"/>
+      <c r="B33" s="74"/>
+      <c r="C33" s="74"/>
+      <c r="D33" s="74"/>
+      <c r="E33" s="74"/>
+      <c r="F33" s="74"/>
+      <c r="G33" s="74"/>
+      <c r="H33" s="74"/>
+      <c r="I33" s="74"/>
+      <c r="J33" s="74"/>
+      <c r="K33" s="74"/>
+      <c r="L33" s="74"/>
+      <c r="M33" s="74"/>
+      <c r="N33" s="74"/>
+      <c r="O33" s="74"/>
       <c r="P33" s="17"/>
       <c r="Q33" s="5"/>
       <c r="R33" s="5"/>
@@ -2795,17 +2795,17 @@
     </row>
     <row r="34" spans="1:25" ht="18" customHeight="1">
       <c r="A34" s="75" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B34" s="75"/>
       <c r="C34" s="75"/>
       <c r="D34" s="75"/>
       <c r="E34" s="75"/>
       <c r="F34" s="61" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G34" s="19" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H34" s="19"/>
       <c r="I34" s="19"/>
@@ -2826,7 +2826,7 @@
       <c r="X34" s="5"/>
       <c r="Y34" s="5"/>
     </row>
-    <row r="35" spans="1:25" ht="15.5" customHeight="1">
+    <row r="35" spans="1:25" ht="15.45" customHeight="1">
       <c r="A35" s="17"/>
       <c r="B35" s="17"/>
       <c r="C35" s="17"/>
@@ -2855,11 +2855,11 @@
     </row>
     <row r="36" spans="1:25" ht="18" customHeight="1">
       <c r="A36" s="75" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B36" s="75"/>
       <c r="C36" s="75" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D36" s="75"/>
       <c r="E36" s="75"/>
@@ -2868,7 +2868,7 @@
       <c r="H36" s="17"/>
       <c r="I36" s="23"/>
       <c r="L36" s="75" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="M36" s="75"/>
       <c r="N36" s="75"/>
@@ -2880,11 +2880,11 @@
     </row>
     <row r="37" spans="1:25" ht="18" customHeight="1">
       <c r="A37" s="75" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B37" s="75"/>
       <c r="C37" s="75" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D37" s="75"/>
       <c r="E37" s="75"/>
@@ -2893,7 +2893,7 @@
       <c r="H37" s="17"/>
       <c r="I37" s="23"/>
       <c r="L37" s="75" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="M37" s="75"/>
       <c r="N37" s="75"/>
@@ -2906,21 +2906,21 @@
     <row r="38" spans="1:25" ht="18" customHeight="1">
       <c r="A38" s="8"/>
       <c r="B38" s="20"/>
-      <c r="C38" s="95" t="s">
-        <v>66</v>
+      <c r="C38" s="78" t="s">
+        <v>65</v>
       </c>
-      <c r="D38" s="95"/>
-      <c r="E38" s="95"/>
+      <c r="D38" s="78"/>
+      <c r="E38" s="78"/>
       <c r="F38" s="23"/>
       <c r="G38" s="23"/>
       <c r="H38" s="23"/>
       <c r="I38" s="23"/>
-      <c r="L38" s="95" t="s">
-        <v>70</v>
+      <c r="L38" s="78" t="s">
+        <v>69</v>
       </c>
-      <c r="M38" s="95"/>
-      <c r="N38" s="95"/>
-      <c r="O38" s="95"/>
+      <c r="M38" s="78"/>
+      <c r="N38" s="78"/>
+      <c r="O38" s="78"/>
       <c r="P38" s="8"/>
       <c r="Q38" s="8"/>
       <c r="R38" s="8"/>
@@ -2929,21 +2929,21 @@
     <row r="39" spans="1:25" ht="18" customHeight="1">
       <c r="A39" s="8"/>
       <c r="B39" s="20"/>
-      <c r="C39" s="95" t="s">
-        <v>67</v>
+      <c r="C39" s="78" t="s">
+        <v>66</v>
       </c>
-      <c r="D39" s="95"/>
-      <c r="E39" s="95"/>
+      <c r="D39" s="78"/>
+      <c r="E39" s="78"/>
       <c r="F39" s="23"/>
       <c r="G39" s="23"/>
       <c r="H39" s="23"/>
       <c r="I39" s="23"/>
-      <c r="L39" s="95" t="s">
-        <v>71</v>
+      <c r="L39" s="78" t="s">
+        <v>70</v>
       </c>
-      <c r="M39" s="95"/>
-      <c r="N39" s="95"/>
-      <c r="O39" s="95"/>
+      <c r="M39" s="78"/>
+      <c r="N39" s="78"/>
+      <c r="O39" s="78"/>
       <c r="P39" s="21"/>
       <c r="Q39" s="21"/>
       <c r="R39" s="21"/>
@@ -3651,7 +3651,7 @@
       <c r="X65" s="5"/>
       <c r="Y65" s="5"/>
     </row>
-    <row r="66" spans="1:25" ht="59" customHeight="1">
+    <row r="66" spans="1:25" ht="58.95" customHeight="1">
       <c r="A66" s="5"/>
       <c r="B66" s="5"/>
       <c r="C66" s="5"/>
@@ -4056,7 +4056,7 @@
       <c r="X80" s="5"/>
       <c r="Y80" s="5"/>
     </row>
-    <row r="81" spans="1:25" ht="46" customHeight="1">
+    <row r="81" spans="1:25" ht="46.05" customHeight="1">
       <c r="A81" s="5"/>
       <c r="B81" s="5"/>
       <c r="C81" s="5"/>
@@ -27810,27 +27810,6 @@
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
   <mergeCells count="37">
-    <mergeCell ref="A21:F21"/>
-    <mergeCell ref="A33:O33"/>
-    <mergeCell ref="A34:E34"/>
-    <mergeCell ref="A36:B36"/>
-    <mergeCell ref="A37:B37"/>
-    <mergeCell ref="A22:F22"/>
-    <mergeCell ref="C38:E38"/>
-    <mergeCell ref="C36:E36"/>
-    <mergeCell ref="H23:O23"/>
-    <mergeCell ref="H24:O28"/>
-    <mergeCell ref="C39:E39"/>
-    <mergeCell ref="C37:E37"/>
-    <mergeCell ref="L38:O38"/>
-    <mergeCell ref="L39:O39"/>
-    <mergeCell ref="K8:M8"/>
-    <mergeCell ref="H15:H16"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="D15:D16"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="F15:F16"/>
     <mergeCell ref="N8:O8"/>
     <mergeCell ref="K9:O9"/>
     <mergeCell ref="L36:O36"/>
@@ -27847,6 +27826,27 @@
     <mergeCell ref="A11:O11"/>
     <mergeCell ref="A12:O12"/>
     <mergeCell ref="A14:O14"/>
+    <mergeCell ref="K8:M8"/>
+    <mergeCell ref="H15:H16"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="D15:D16"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="F15:F16"/>
+    <mergeCell ref="C38:E38"/>
+    <mergeCell ref="C36:E36"/>
+    <mergeCell ref="H23:O23"/>
+    <mergeCell ref="H24:O28"/>
+    <mergeCell ref="C39:E39"/>
+    <mergeCell ref="C37:E37"/>
+    <mergeCell ref="L38:O38"/>
+    <mergeCell ref="L39:O39"/>
+    <mergeCell ref="A21:F21"/>
+    <mergeCell ref="A33:O33"/>
+    <mergeCell ref="A34:E34"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="A22:F22"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>

</xml_diff>

<commit_message>
feat: add Єдиний Акт Списання (EAS) report with cross-report conversions
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Mil.Paperwork.Domain/Templates/ResidualValueReportTemplate.xlsx
+++ b/Mil.Paperwork.Domain/Templates/ResidualValueReportTemplate.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr codeName="Workbook_______"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\Projects\Mil.Paperwork.WriteOff\Mil.Paperwork.Domain\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7E80A4F-BCC2-4309-9075-5A94E82FA98C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FB48131-4D26-4D9A-894C-E6B05505CFC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-9165" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Відомість" sheetId="1" r:id="rId1"/>
@@ -299,10 +299,10 @@
     <t>[COMMISSION_PERSON3_NAME]</t>
   </si>
   <si>
-    <t>Командир військової частини [MIL_UNIT]</t>
+    <t>"____" __________ 2026 року</t>
   </si>
   <si>
-    <t>"____" __________ 2026 року</t>
+    <t>[COMM_POSITION] [MIL_UNIT]</t>
   </si>
 </sst>
 </file>
@@ -918,7 +918,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="102">
+  <cellXfs count="101">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1012,7 +1012,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1119,62 +1118,13 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1198,8 +1148,57 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1999,10 +1998,10 @@
       <c r="Y2" s="5"/>
     </row>
     <row r="3" spans="1:25" ht="12.75" customHeight="1">
-      <c r="A3" s="93" t="s">
+      <c r="A3" s="75" t="s">
         <v>62</v>
       </c>
-      <c r="B3" s="94"/>
+      <c r="B3" s="76"/>
       <c r="C3" s="5"/>
       <c r="D3" s="5"/>
       <c r="E3" s="5"/>
@@ -2028,14 +2027,14 @@
       <c r="Y3" s="5"/>
     </row>
     <row r="4" spans="1:25" ht="12.75" customHeight="1">
-      <c r="A4" s="95" t="s">
+      <c r="A4" s="77" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="94"/>
-      <c r="C4" s="97" t="s">
+      <c r="B4" s="76"/>
+      <c r="C4" s="79" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="98"/>
+      <c r="D4" s="80"/>
       <c r="E4" s="27"/>
       <c r="F4" s="5"/>
       <c r="G4" s="5"/>
@@ -2086,19 +2085,19 @@
       <c r="Y5" s="5"/>
     </row>
     <row r="6" spans="1:25" ht="18" customHeight="1">
-      <c r="A6" s="96"/>
-      <c r="B6" s="94"/>
+      <c r="A6" s="78"/>
+      <c r="B6" s="76"/>
       <c r="C6" s="7"/>
       <c r="D6" s="7"/>
       <c r="E6" s="7"/>
       <c r="F6" s="7"/>
-      <c r="K6" s="92" t="s">
+      <c r="K6" s="73" t="s">
         <v>1</v>
       </c>
-      <c r="L6" s="92"/>
-      <c r="M6" s="92"/>
-      <c r="N6" s="92"/>
-      <c r="O6" s="92"/>
+      <c r="L6" s="73"/>
+      <c r="M6" s="73"/>
+      <c r="N6" s="73"/>
+      <c r="O6" s="73"/>
       <c r="P6" s="20"/>
     </row>
     <row r="7" spans="1:25" ht="18">
@@ -2107,13 +2106,13 @@
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
       <c r="E7" s="7"/>
-      <c r="K7" s="75" t="s">
-        <v>71</v>
+      <c r="K7" s="74" t="s">
+        <v>72</v>
       </c>
-      <c r="L7" s="92"/>
-      <c r="M7" s="92"/>
-      <c r="N7" s="92"/>
-      <c r="O7" s="92"/>
+      <c r="L7" s="73"/>
+      <c r="M7" s="73"/>
+      <c r="N7" s="73"/>
+      <c r="O7" s="73"/>
       <c r="P7" s="20"/>
     </row>
     <row r="8" spans="1:25" ht="18" customHeight="1">
@@ -2122,15 +2121,15 @@
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
       <c r="E8" s="7"/>
-      <c r="K8" s="81" t="s">
+      <c r="K8" s="86" t="s">
         <v>60</v>
       </c>
-      <c r="L8" s="81"/>
-      <c r="M8" s="81"/>
-      <c r="N8" s="91" t="s">
+      <c r="L8" s="86"/>
+      <c r="M8" s="86"/>
+      <c r="N8" s="72" t="s">
         <v>61</v>
       </c>
-      <c r="O8" s="91"/>
+      <c r="O8" s="72"/>
       <c r="P8" s="8"/>
     </row>
     <row r="9" spans="1:25" ht="24.75" customHeight="1">
@@ -2139,13 +2138,13 @@
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
       <c r="E9" s="7"/>
-      <c r="K9" s="92" t="s">
-        <v>72</v>
+      <c r="K9" s="73" t="s">
+        <v>71</v>
       </c>
-      <c r="L9" s="92"/>
-      <c r="M9" s="92"/>
-      <c r="N9" s="92"/>
-      <c r="O9" s="92"/>
+      <c r="L9" s="73"/>
+      <c r="M9" s="73"/>
+      <c r="N9" s="73"/>
+      <c r="O9" s="73"/>
       <c r="P9" s="20"/>
     </row>
     <row r="10" spans="1:25" ht="18" customHeight="1">
@@ -2166,23 +2165,23 @@
       <c r="Y10" s="8"/>
     </row>
     <row r="11" spans="1:25" ht="18" customHeight="1">
-      <c r="A11" s="101" t="s">
+      <c r="A11" s="85" t="s">
         <v>2</v>
       </c>
-      <c r="B11" s="101"/>
-      <c r="C11" s="101"/>
-      <c r="D11" s="101"/>
-      <c r="E11" s="101"/>
-      <c r="F11" s="101"/>
-      <c r="G11" s="101"/>
-      <c r="H11" s="101"/>
-      <c r="I11" s="101"/>
-      <c r="J11" s="101"/>
-      <c r="K11" s="101"/>
-      <c r="L11" s="101"/>
-      <c r="M11" s="101"/>
-      <c r="N11" s="101"/>
-      <c r="O11" s="101"/>
+      <c r="B11" s="85"/>
+      <c r="C11" s="85"/>
+      <c r="D11" s="85"/>
+      <c r="E11" s="85"/>
+      <c r="F11" s="85"/>
+      <c r="G11" s="85"/>
+      <c r="H11" s="85"/>
+      <c r="I11" s="85"/>
+      <c r="J11" s="85"/>
+      <c r="K11" s="85"/>
+      <c r="L11" s="85"/>
+      <c r="M11" s="85"/>
+      <c r="N11" s="85"/>
+      <c r="O11" s="85"/>
       <c r="P11" s="8"/>
       <c r="Q11" s="8"/>
       <c r="R11" s="8"/>
@@ -2195,86 +2194,86 @@
       <c r="Y11" s="8"/>
     </row>
     <row r="12" spans="1:25" ht="18" customHeight="1">
-      <c r="A12" s="100" t="s">
+      <c r="A12" s="82" t="s">
         <v>32</v>
       </c>
-      <c r="B12" s="100"/>
-      <c r="C12" s="100"/>
-      <c r="D12" s="100"/>
-      <c r="E12" s="100"/>
-      <c r="F12" s="100"/>
-      <c r="G12" s="100"/>
-      <c r="H12" s="100"/>
-      <c r="I12" s="100"/>
-      <c r="J12" s="100"/>
-      <c r="K12" s="100"/>
-      <c r="L12" s="100"/>
-      <c r="M12" s="100"/>
-      <c r="N12" s="100"/>
-      <c r="O12" s="100"/>
+      <c r="B12" s="82"/>
+      <c r="C12" s="82"/>
+      <c r="D12" s="82"/>
+      <c r="E12" s="82"/>
+      <c r="F12" s="82"/>
+      <c r="G12" s="82"/>
+      <c r="H12" s="82"/>
+      <c r="I12" s="82"/>
+      <c r="J12" s="82"/>
+      <c r="K12" s="82"/>
+      <c r="L12" s="82"/>
+      <c r="M12" s="82"/>
+      <c r="N12" s="82"/>
+      <c r="O12" s="82"/>
       <c r="P12" s="8"/>
     </row>
-    <row r="13" spans="1:25" s="37" customFormat="1" ht="18" customHeight="1">
-      <c r="A13" s="100" t="s">
+    <row r="13" spans="1:25" ht="18" customHeight="1">
+      <c r="A13" s="82" t="s">
         <v>58</v>
       </c>
-      <c r="B13" s="100"/>
-      <c r="C13" s="100"/>
-      <c r="D13" s="100"/>
-      <c r="E13" s="100"/>
-      <c r="F13" s="100"/>
-      <c r="G13" s="100"/>
-      <c r="H13" s="100"/>
-      <c r="I13" s="100"/>
-      <c r="J13" s="100"/>
-      <c r="K13" s="100"/>
-      <c r="L13" s="100"/>
-      <c r="M13" s="100"/>
-      <c r="N13" s="100"/>
-      <c r="O13" s="100"/>
+      <c r="B13" s="82"/>
+      <c r="C13" s="82"/>
+      <c r="D13" s="82"/>
+      <c r="E13" s="82"/>
+      <c r="F13" s="82"/>
+      <c r="G13" s="82"/>
+      <c r="H13" s="82"/>
+      <c r="I13" s="82"/>
+      <c r="J13" s="82"/>
+      <c r="K13" s="82"/>
+      <c r="L13" s="82"/>
+      <c r="M13" s="82"/>
+      <c r="N13" s="82"/>
+      <c r="O13" s="82"/>
       <c r="P13" s="8"/>
     </row>
     <row r="14" spans="1:25" ht="18" customHeight="1">
-      <c r="A14" s="101"/>
-      <c r="B14" s="101"/>
-      <c r="C14" s="101"/>
-      <c r="D14" s="101"/>
-      <c r="E14" s="101"/>
-      <c r="F14" s="101"/>
-      <c r="G14" s="101"/>
-      <c r="H14" s="101"/>
-      <c r="I14" s="101"/>
-      <c r="J14" s="101"/>
-      <c r="K14" s="101"/>
-      <c r="L14" s="101"/>
-      <c r="M14" s="101"/>
-      <c r="N14" s="101"/>
-      <c r="O14" s="101"/>
+      <c r="A14" s="85"/>
+      <c r="B14" s="85"/>
+      <c r="C14" s="85"/>
+      <c r="D14" s="85"/>
+      <c r="E14" s="85"/>
+      <c r="F14" s="85"/>
+      <c r="G14" s="85"/>
+      <c r="H14" s="85"/>
+      <c r="I14" s="85"/>
+      <c r="J14" s="85"/>
+      <c r="K14" s="85"/>
+      <c r="L14" s="85"/>
+      <c r="M14" s="85"/>
+      <c r="N14" s="85"/>
+      <c r="O14" s="85"/>
       <c r="P14" s="8"/>
     </row>
     <row r="15" spans="1:25" ht="67.95" customHeight="1">
-      <c r="A15" s="84" t="s">
+      <c r="A15" s="83" t="s">
         <v>3</v>
       </c>
-      <c r="B15" s="84" t="s">
+      <c r="B15" s="83" t="s">
         <v>4</v>
       </c>
-      <c r="C15" s="84" t="s">
+      <c r="C15" s="83" t="s">
         <v>5</v>
       </c>
-      <c r="D15" s="87" t="s">
+      <c r="D15" s="90" t="s">
         <v>6</v>
       </c>
-      <c r="E15" s="99" t="s">
+      <c r="E15" s="81" t="s">
         <v>33</v>
       </c>
-      <c r="F15" s="89" t="s">
+      <c r="F15" s="92" t="s">
         <v>21</v>
       </c>
-      <c r="G15" s="84" t="s">
+      <c r="G15" s="83" t="s">
         <v>59</v>
       </c>
-      <c r="H15" s="82" t="s">
+      <c r="H15" s="87" t="s">
         <v>7</v>
       </c>
       <c r="I15" s="28"/>
@@ -2283,14 +2282,14 @@
       <c r="O15" s="10"/>
     </row>
     <row r="16" spans="1:25" ht="24" customHeight="1">
-      <c r="A16" s="85"/>
-      <c r="B16" s="86"/>
-      <c r="C16" s="86"/>
-      <c r="D16" s="88"/>
-      <c r="E16" s="99"/>
-      <c r="F16" s="90"/>
-      <c r="G16" s="86"/>
-      <c r="H16" s="83"/>
+      <c r="A16" s="89"/>
+      <c r="B16" s="84"/>
+      <c r="C16" s="84"/>
+      <c r="D16" s="91"/>
+      <c r="E16" s="81"/>
+      <c r="F16" s="93"/>
+      <c r="G16" s="84"/>
+      <c r="H16" s="88"/>
       <c r="I16" s="16"/>
       <c r="M16" s="28"/>
       <c r="N16" s="9"/>
@@ -2309,7 +2308,7 @@
       <c r="D17" s="35">
         <v>4</v>
       </c>
-      <c r="E17" s="38">
+      <c r="E17" s="37">
         <v>5</v>
       </c>
       <c r="F17" s="1">
@@ -2330,16 +2329,16 @@
       <c r="A18" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B18" s="65" t="s">
+      <c r="B18" s="64" t="s">
         <v>14</v>
       </c>
-      <c r="C18" s="66" t="s">
+      <c r="C18" s="65" t="s">
         <v>15</v>
       </c>
       <c r="D18" s="36" t="s">
         <v>16</v>
       </c>
-      <c r="E18" s="67" t="s">
+      <c r="E18" s="66" t="s">
         <v>17</v>
       </c>
       <c r="F18" s="36" t="s">
@@ -2374,15 +2373,15 @@
       </c>
     </row>
     <row r="19" spans="1:25" ht="15.6">
-      <c r="A19" s="63"/>
-      <c r="B19" s="68"/>
-      <c r="C19" s="69"/>
-      <c r="D19" s="70"/>
-      <c r="E19" s="71">
+      <c r="A19" s="62"/>
+      <c r="B19" s="67"/>
+      <c r="C19" s="68"/>
+      <c r="D19" s="69"/>
+      <c r="E19" s="70">
         <v>100000</v>
       </c>
-      <c r="F19" s="72"/>
-      <c r="G19" s="64">
+      <c r="F19" s="71"/>
+      <c r="G19" s="63">
         <f>ROUND(E19*F19,2)</f>
         <v>0</v>
       </c>
@@ -2413,15 +2412,15 @@
       <c r="O20" s="16"/>
       <c r="P20" s="5"/>
     </row>
-    <row r="21" spans="1:25" s="37" customFormat="1" ht="15" customHeight="1">
-      <c r="A21" s="73" t="s">
+    <row r="21" spans="1:25" ht="15" customHeight="1">
+      <c r="A21" s="97" t="s">
         <v>51</v>
       </c>
-      <c r="B21" s="73"/>
-      <c r="C21" s="73"/>
-      <c r="D21" s="73"/>
-      <c r="E21" s="73"/>
-      <c r="F21" s="73"/>
+      <c r="B21" s="97"/>
+      <c r="C21" s="97"/>
+      <c r="D21" s="97"/>
+      <c r="E21" s="97"/>
+      <c r="F21" s="97"/>
       <c r="G21" s="12"/>
       <c r="H21" s="15"/>
       <c r="I21" s="13"/>
@@ -2434,266 +2433,266 @@
       <c r="P21" s="5"/>
     </row>
     <row r="22" spans="1:25" ht="18.600000000000001" thickBot="1">
-      <c r="A22" s="76" t="s">
+      <c r="A22" s="99" t="s">
         <v>43</v>
       </c>
-      <c r="B22" s="77"/>
-      <c r="C22" s="77"/>
-      <c r="D22" s="77"/>
-      <c r="E22" s="77"/>
-      <c r="F22" s="77"/>
-      <c r="G22" s="53"/>
-      <c r="H22" s="53"/>
-      <c r="I22" s="53"/>
-      <c r="J22" s="53"/>
-      <c r="K22" s="53"/>
-      <c r="L22" s="53"/>
-      <c r="M22" s="53"/>
-      <c r="N22" s="54"/>
-      <c r="O22" s="54"/>
+      <c r="B22" s="100"/>
+      <c r="C22" s="100"/>
+      <c r="D22" s="100"/>
+      <c r="E22" s="100"/>
+      <c r="F22" s="100"/>
+      <c r="G22" s="52"/>
+      <c r="H22" s="52"/>
+      <c r="I22" s="52"/>
+      <c r="J22" s="52"/>
+      <c r="K22" s="52"/>
+      <c r="L22" s="52"/>
+      <c r="M22" s="52"/>
+      <c r="N22" s="53"/>
+      <c r="O22" s="53"/>
     </row>
     <row r="23" spans="1:25" ht="66">
-      <c r="A23" s="55" t="s">
+      <c r="A23" s="54" t="s">
         <v>8</v>
       </c>
-      <c r="B23" s="39" t="s">
+      <c r="B23" s="38" t="s">
         <v>9</v>
       </c>
-      <c r="C23" s="40" t="s">
+      <c r="C23" s="39" t="s">
         <v>34</v>
       </c>
-      <c r="D23" s="40" t="s">
+      <c r="D23" s="39" t="s">
         <v>35</v>
       </c>
-      <c r="E23" s="39" t="s">
+      <c r="E23" s="38" t="s">
         <v>10</v>
       </c>
-      <c r="F23" s="41" t="s">
+      <c r="F23" s="40" t="s">
         <v>11</v>
       </c>
-      <c r="G23" s="56"/>
-      <c r="H23" s="79" t="s">
+      <c r="G23" s="55"/>
+      <c r="H23" s="95" t="s">
         <v>57</v>
       </c>
-      <c r="I23" s="79"/>
-      <c r="J23" s="79"/>
-      <c r="K23" s="79"/>
-      <c r="L23" s="79"/>
-      <c r="M23" s="79"/>
-      <c r="N23" s="79"/>
-      <c r="O23" s="79"/>
+      <c r="I23" s="95"/>
+      <c r="J23" s="95"/>
+      <c r="K23" s="95"/>
+      <c r="L23" s="95"/>
+      <c r="M23" s="95"/>
+      <c r="N23" s="95"/>
+      <c r="O23" s="95"/>
       <c r="P23" s="8"/>
     </row>
     <row r="24" spans="1:25" ht="15.45" customHeight="1">
-      <c r="A24" s="57" t="s">
+      <c r="A24" s="56" t="s">
         <v>44</v>
       </c>
-      <c r="B24" s="42" t="s">
+      <c r="B24" s="41" t="s">
         <v>36</v>
       </c>
-      <c r="C24" s="43"/>
-      <c r="D24" s="44">
+      <c r="C24" s="42"/>
+      <c r="D24" s="43">
         <f>ROUND(C24*$D$19,2)</f>
         <v>0</v>
       </c>
-      <c r="E24" s="45">
+      <c r="E24" s="44">
         <v>0</v>
       </c>
-      <c r="F24" s="46">
+      <c r="F24" s="45">
         <f>D24*E24</f>
         <v>0</v>
       </c>
-      <c r="G24" s="56"/>
-      <c r="H24" s="80" t="s">
+      <c r="G24" s="55"/>
+      <c r="H24" s="96" t="s">
         <v>56</v>
       </c>
-      <c r="I24" s="80"/>
-      <c r="J24" s="80"/>
-      <c r="K24" s="80"/>
-      <c r="L24" s="80"/>
-      <c r="M24" s="80"/>
-      <c r="N24" s="80"/>
-      <c r="O24" s="80"/>
+      <c r="I24" s="96"/>
+      <c r="J24" s="96"/>
+      <c r="K24" s="96"/>
+      <c r="L24" s="96"/>
+      <c r="M24" s="96"/>
+      <c r="N24" s="96"/>
+      <c r="O24" s="96"/>
       <c r="P24" s="5"/>
     </row>
     <row r="25" spans="1:25" ht="18" customHeight="1">
-      <c r="A25" s="57" t="s">
+      <c r="A25" s="56" t="s">
         <v>45</v>
       </c>
-      <c r="B25" s="42" t="s">
+      <c r="B25" s="41" t="s">
         <v>37</v>
       </c>
-      <c r="C25" s="43"/>
-      <c r="D25" s="44">
+      <c r="C25" s="42"/>
+      <c r="D25" s="43">
         <f t="shared" ref="D25:D30" si="0">ROUND(C25*$D$19,2)</f>
         <v>0</v>
       </c>
-      <c r="E25" s="45">
+      <c r="E25" s="44">
         <v>0</v>
       </c>
-      <c r="F25" s="46">
+      <c r="F25" s="45">
         <f t="shared" ref="F25:F30" si="1">D25*E25</f>
         <v>0</v>
       </c>
-      <c r="G25" s="56"/>
-      <c r="H25" s="80"/>
-      <c r="I25" s="80"/>
-      <c r="J25" s="80"/>
-      <c r="K25" s="80"/>
-      <c r="L25" s="80"/>
-      <c r="M25" s="80"/>
-      <c r="N25" s="80"/>
-      <c r="O25" s="80"/>
+      <c r="G25" s="55"/>
+      <c r="H25" s="96"/>
+      <c r="I25" s="96"/>
+      <c r="J25" s="96"/>
+      <c r="K25" s="96"/>
+      <c r="L25" s="96"/>
+      <c r="M25" s="96"/>
+      <c r="N25" s="96"/>
+      <c r="O25" s="96"/>
       <c r="P25" s="5"/>
     </row>
     <row r="26" spans="1:25" ht="15.45" customHeight="1">
-      <c r="A26" s="57" t="s">
+      <c r="A26" s="56" t="s">
         <v>46</v>
       </c>
-      <c r="B26" s="42" t="s">
+      <c r="B26" s="41" t="s">
         <v>38</v>
       </c>
-      <c r="C26" s="43"/>
-      <c r="D26" s="44">
+      <c r="C26" s="42"/>
+      <c r="D26" s="43">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="E26" s="45">
+      <c r="E26" s="44">
         <v>0</v>
       </c>
-      <c r="F26" s="46">
+      <c r="F26" s="45">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="G26" s="56"/>
-      <c r="H26" s="80"/>
-      <c r="I26" s="80"/>
-      <c r="J26" s="80"/>
-      <c r="K26" s="80"/>
-      <c r="L26" s="80"/>
-      <c r="M26" s="80"/>
-      <c r="N26" s="80"/>
-      <c r="O26" s="80"/>
+      <c r="G26" s="55"/>
+      <c r="H26" s="96"/>
+      <c r="I26" s="96"/>
+      <c r="J26" s="96"/>
+      <c r="K26" s="96"/>
+      <c r="L26" s="96"/>
+      <c r="M26" s="96"/>
+      <c r="N26" s="96"/>
+      <c r="O26" s="96"/>
       <c r="P26" s="5"/>
     </row>
     <row r="27" spans="1:25" ht="15.45" customHeight="1">
-      <c r="A27" s="57" t="s">
+      <c r="A27" s="56" t="s">
         <v>47</v>
       </c>
-      <c r="B27" s="42" t="s">
+      <c r="B27" s="41" t="s">
         <v>39</v>
       </c>
-      <c r="C27" s="43"/>
-      <c r="D27" s="44">
+      <c r="C27" s="42"/>
+      <c r="D27" s="43">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="E27" s="45">
+      <c r="E27" s="44">
         <v>0</v>
       </c>
-      <c r="F27" s="46">
+      <c r="F27" s="45">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="G27" s="56"/>
-      <c r="H27" s="80"/>
-      <c r="I27" s="80"/>
-      <c r="J27" s="80"/>
-      <c r="K27" s="80"/>
-      <c r="L27" s="80"/>
-      <c r="M27" s="80"/>
-      <c r="N27" s="80"/>
-      <c r="O27" s="80"/>
+      <c r="G27" s="55"/>
+      <c r="H27" s="96"/>
+      <c r="I27" s="96"/>
+      <c r="J27" s="96"/>
+      <c r="K27" s="96"/>
+      <c r="L27" s="96"/>
+      <c r="M27" s="96"/>
+      <c r="N27" s="96"/>
+      <c r="O27" s="96"/>
       <c r="P27" s="5"/>
     </row>
     <row r="28" spans="1:25" ht="15.45" customHeight="1">
-      <c r="A28" s="57" t="s">
+      <c r="A28" s="56" t="s">
         <v>48</v>
       </c>
-      <c r="B28" s="42" t="s">
+      <c r="B28" s="41" t="s">
         <v>40</v>
       </c>
-      <c r="C28" s="47"/>
-      <c r="D28" s="44">
+      <c r="C28" s="46"/>
+      <c r="D28" s="43">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="E28" s="45">
+      <c r="E28" s="44">
         <v>5</v>
       </c>
-      <c r="F28" s="46">
+      <c r="F28" s="45">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="G28" s="56"/>
-      <c r="H28" s="80"/>
-      <c r="I28" s="80"/>
-      <c r="J28" s="80"/>
-      <c r="K28" s="80"/>
-      <c r="L28" s="80"/>
-      <c r="M28" s="80"/>
-      <c r="N28" s="80"/>
-      <c r="O28" s="80"/>
+      <c r="G28" s="55"/>
+      <c r="H28" s="96"/>
+      <c r="I28" s="96"/>
+      <c r="J28" s="96"/>
+      <c r="K28" s="96"/>
+      <c r="L28" s="96"/>
+      <c r="M28" s="96"/>
+      <c r="N28" s="96"/>
+      <c r="O28" s="96"/>
       <c r="P28" s="5"/>
     </row>
     <row r="29" spans="1:25" ht="15" customHeight="1">
-      <c r="A29" s="58" t="s">
+      <c r="A29" s="57" t="s">
         <v>49</v>
       </c>
-      <c r="B29" s="42" t="s">
+      <c r="B29" s="41" t="s">
         <v>41</v>
       </c>
-      <c r="C29" s="47"/>
-      <c r="D29" s="44">
+      <c r="C29" s="46"/>
+      <c r="D29" s="43">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="E29" s="62">
+      <c r="E29" s="61">
         <v>45</v>
       </c>
-      <c r="F29" s="46">
+      <c r="F29" s="45">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="G29" s="56"/>
-      <c r="H29" s="56"/>
-      <c r="I29" s="59"/>
-      <c r="J29" s="59"/>
-      <c r="K29" s="59"/>
-      <c r="L29" s="59"/>
-      <c r="M29" s="59"/>
-      <c r="N29" s="59"/>
-      <c r="O29" s="59"/>
+      <c r="G29" s="55"/>
+      <c r="H29" s="55"/>
+      <c r="I29" s="58"/>
+      <c r="J29" s="58"/>
+      <c r="K29" s="58"/>
+      <c r="L29" s="58"/>
+      <c r="M29" s="58"/>
+      <c r="N29" s="58"/>
+      <c r="O29" s="58"/>
       <c r="P29" s="5"/>
     </row>
     <row r="30" spans="1:25" ht="15" customHeight="1">
-      <c r="A30" s="58" t="s">
+      <c r="A30" s="57" t="s">
         <v>50</v>
       </c>
-      <c r="B30" s="42" t="s">
+      <c r="B30" s="41" t="s">
         <v>42</v>
       </c>
-      <c r="C30" s="47"/>
-      <c r="D30" s="44">
+      <c r="C30" s="46"/>
+      <c r="D30" s="43">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="E30" s="62">
+      <c r="E30" s="61">
         <v>270</v>
       </c>
-      <c r="F30" s="46">
+      <c r="F30" s="45">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="G30" s="56"/>
-      <c r="H30" s="56"/>
-      <c r="I30" s="59"/>
-      <c r="J30" s="59"/>
-      <c r="K30" s="59"/>
-      <c r="L30" s="59"/>
-      <c r="M30" s="59"/>
-      <c r="N30" s="59"/>
-      <c r="O30" s="59"/>
+      <c r="G30" s="55"/>
+      <c r="H30" s="55"/>
+      <c r="I30" s="58"/>
+      <c r="J30" s="58"/>
+      <c r="K30" s="58"/>
+      <c r="L30" s="58"/>
+      <c r="M30" s="58"/>
+      <c r="N30" s="58"/>
+      <c r="O30" s="58"/>
       <c r="P30" s="5"/>
       <c r="Q30" s="5"/>
       <c r="R30" s="5"/>
@@ -2706,26 +2705,26 @@
       <c r="Y30" s="5"/>
     </row>
     <row r="31" spans="1:25" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A31" s="60"/>
-      <c r="B31" s="48" t="s">
+      <c r="A31" s="59"/>
+      <c r="B31" s="47" t="s">
         <v>12</v>
       </c>
-      <c r="C31" s="49"/>
-      <c r="D31" s="50"/>
-      <c r="E31" s="51"/>
-      <c r="F31" s="52">
+      <c r="C31" s="48"/>
+      <c r="D31" s="49"/>
+      <c r="E31" s="50"/>
+      <c r="F31" s="51">
         <f>SUM(F24:F30)</f>
         <v>0</v>
       </c>
-      <c r="G31" s="56"/>
-      <c r="H31" s="56"/>
-      <c r="I31" s="59"/>
-      <c r="J31" s="59"/>
-      <c r="K31" s="59"/>
-      <c r="L31" s="59"/>
-      <c r="M31" s="59"/>
-      <c r="N31" s="59"/>
-      <c r="O31" s="59"/>
+      <c r="G31" s="55"/>
+      <c r="H31" s="55"/>
+      <c r="I31" s="58"/>
+      <c r="J31" s="58"/>
+      <c r="K31" s="58"/>
+      <c r="L31" s="58"/>
+      <c r="M31" s="58"/>
+      <c r="N31" s="58"/>
+      <c r="O31" s="58"/>
       <c r="P31" s="5"/>
       <c r="Q31" s="5"/>
       <c r="R31" s="5"/>
@@ -2765,23 +2764,23 @@
       <c r="Y32" s="5"/>
     </row>
     <row r="33" spans="1:25" ht="18">
-      <c r="A33" s="74" t="s">
+      <c r="A33" s="98" t="s">
         <v>55</v>
       </c>
-      <c r="B33" s="74"/>
-      <c r="C33" s="74"/>
-      <c r="D33" s="74"/>
-      <c r="E33" s="74"/>
-      <c r="F33" s="74"/>
-      <c r="G33" s="74"/>
-      <c r="H33" s="74"/>
-      <c r="I33" s="74"/>
-      <c r="J33" s="74"/>
-      <c r="K33" s="74"/>
-      <c r="L33" s="74"/>
-      <c r="M33" s="74"/>
-      <c r="N33" s="74"/>
-      <c r="O33" s="74"/>
+      <c r="B33" s="98"/>
+      <c r="C33" s="98"/>
+      <c r="D33" s="98"/>
+      <c r="E33" s="98"/>
+      <c r="F33" s="98"/>
+      <c r="G33" s="98"/>
+      <c r="H33" s="98"/>
+      <c r="I33" s="98"/>
+      <c r="J33" s="98"/>
+      <c r="K33" s="98"/>
+      <c r="L33" s="98"/>
+      <c r="M33" s="98"/>
+      <c r="N33" s="98"/>
+      <c r="O33" s="98"/>
       <c r="P33" s="17"/>
       <c r="Q33" s="5"/>
       <c r="R33" s="5"/>
@@ -2794,14 +2793,14 @@
       <c r="Y33" s="5"/>
     </row>
     <row r="34" spans="1:25" ht="18" customHeight="1">
-      <c r="A34" s="75" t="s">
+      <c r="A34" s="74" t="s">
         <v>52</v>
       </c>
-      <c r="B34" s="75"/>
-      <c r="C34" s="75"/>
-      <c r="D34" s="75"/>
-      <c r="E34" s="75"/>
-      <c r="F34" s="61" t="s">
+      <c r="B34" s="74"/>
+      <c r="C34" s="74"/>
+      <c r="D34" s="74"/>
+      <c r="E34" s="74"/>
+      <c r="F34" s="60" t="s">
         <v>54</v>
       </c>
       <c r="G34" s="19" t="s">
@@ -2854,50 +2853,50 @@
       <c r="Y35" s="5"/>
     </row>
     <row r="36" spans="1:25" ht="18" customHeight="1">
-      <c r="A36" s="75" t="s">
+      <c r="A36" s="74" t="s">
         <v>31</v>
       </c>
-      <c r="B36" s="75"/>
-      <c r="C36" s="75" t="s">
+      <c r="B36" s="74"/>
+      <c r="C36" s="74" t="s">
         <v>64</v>
       </c>
-      <c r="D36" s="75"/>
-      <c r="E36" s="75"/>
+      <c r="D36" s="74"/>
+      <c r="E36" s="74"/>
       <c r="F36" s="17"/>
       <c r="G36" s="17"/>
       <c r="H36" s="17"/>
       <c r="I36" s="23"/>
-      <c r="L36" s="75" t="s">
+      <c r="L36" s="74" t="s">
         <v>67</v>
       </c>
-      <c r="M36" s="75"/>
-      <c r="N36" s="75"/>
-      <c r="O36" s="75"/>
+      <c r="M36" s="74"/>
+      <c r="N36" s="74"/>
+      <c r="O36" s="74"/>
       <c r="P36" s="8"/>
       <c r="Q36" s="8"/>
       <c r="R36" s="5"/>
       <c r="Y36" s="5"/>
     </row>
     <row r="37" spans="1:25" ht="18" customHeight="1">
-      <c r="A37" s="75" t="s">
+      <c r="A37" s="74" t="s">
         <v>22</v>
       </c>
-      <c r="B37" s="75"/>
-      <c r="C37" s="75" t="s">
+      <c r="B37" s="74"/>
+      <c r="C37" s="74" t="s">
         <v>63</v>
       </c>
-      <c r="D37" s="75"/>
-      <c r="E37" s="75"/>
+      <c r="D37" s="74"/>
+      <c r="E37" s="74"/>
       <c r="F37" s="17"/>
       <c r="G37" s="17"/>
       <c r="H37" s="17"/>
       <c r="I37" s="23"/>
-      <c r="L37" s="75" t="s">
+      <c r="L37" s="74" t="s">
         <v>68</v>
       </c>
-      <c r="M37" s="75"/>
-      <c r="N37" s="75"/>
-      <c r="O37" s="75"/>
+      <c r="M37" s="74"/>
+      <c r="N37" s="74"/>
+      <c r="O37" s="74"/>
       <c r="P37" s="8"/>
       <c r="Q37" s="8"/>
       <c r="R37" s="8"/>
@@ -2906,21 +2905,21 @@
     <row r="38" spans="1:25" ht="18" customHeight="1">
       <c r="A38" s="8"/>
       <c r="B38" s="20"/>
-      <c r="C38" s="78" t="s">
+      <c r="C38" s="94" t="s">
         <v>65</v>
       </c>
-      <c r="D38" s="78"/>
-      <c r="E38" s="78"/>
+      <c r="D38" s="94"/>
+      <c r="E38" s="94"/>
       <c r="F38" s="23"/>
       <c r="G38" s="23"/>
       <c r="H38" s="23"/>
       <c r="I38" s="23"/>
-      <c r="L38" s="78" t="s">
+      <c r="L38" s="94" t="s">
         <v>69</v>
       </c>
-      <c r="M38" s="78"/>
-      <c r="N38" s="78"/>
-      <c r="O38" s="78"/>
+      <c r="M38" s="94"/>
+      <c r="N38" s="94"/>
+      <c r="O38" s="94"/>
       <c r="P38" s="8"/>
       <c r="Q38" s="8"/>
       <c r="R38" s="8"/>
@@ -2929,21 +2928,21 @@
     <row r="39" spans="1:25" ht="18" customHeight="1">
       <c r="A39" s="8"/>
       <c r="B39" s="20"/>
-      <c r="C39" s="78" t="s">
+      <c r="C39" s="94" t="s">
         <v>66</v>
       </c>
-      <c r="D39" s="78"/>
-      <c r="E39" s="78"/>
+      <c r="D39" s="94"/>
+      <c r="E39" s="94"/>
       <c r="F39" s="23"/>
       <c r="G39" s="23"/>
       <c r="H39" s="23"/>
       <c r="I39" s="23"/>
-      <c r="L39" s="78" t="s">
+      <c r="L39" s="94" t="s">
         <v>70</v>
       </c>
-      <c r="M39" s="78"/>
-      <c r="N39" s="78"/>
-      <c r="O39" s="78"/>
+      <c r="M39" s="94"/>
+      <c r="N39" s="94"/>
+      <c r="O39" s="94"/>
       <c r="P39" s="21"/>
       <c r="Q39" s="21"/>
       <c r="R39" s="21"/>
@@ -27810,6 +27809,27 @@
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
   <mergeCells count="37">
+    <mergeCell ref="A21:F21"/>
+    <mergeCell ref="A33:O33"/>
+    <mergeCell ref="A34:E34"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="A22:F22"/>
+    <mergeCell ref="C38:E38"/>
+    <mergeCell ref="C36:E36"/>
+    <mergeCell ref="H23:O23"/>
+    <mergeCell ref="H24:O28"/>
+    <mergeCell ref="C39:E39"/>
+    <mergeCell ref="C37:E37"/>
+    <mergeCell ref="L38:O38"/>
+    <mergeCell ref="L39:O39"/>
+    <mergeCell ref="K8:M8"/>
+    <mergeCell ref="H15:H16"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="D15:D16"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="F15:F16"/>
     <mergeCell ref="N8:O8"/>
     <mergeCell ref="K9:O9"/>
     <mergeCell ref="L36:O36"/>
@@ -27826,27 +27846,6 @@
     <mergeCell ref="A11:O11"/>
     <mergeCell ref="A12:O12"/>
     <mergeCell ref="A14:O14"/>
-    <mergeCell ref="K8:M8"/>
-    <mergeCell ref="H15:H16"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="D15:D16"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="F15:F16"/>
-    <mergeCell ref="C38:E38"/>
-    <mergeCell ref="C36:E36"/>
-    <mergeCell ref="H23:O23"/>
-    <mergeCell ref="H24:O28"/>
-    <mergeCell ref="C39:E39"/>
-    <mergeCell ref="C37:E37"/>
-    <mergeCell ref="L38:O38"/>
-    <mergeCell ref="L39:O39"/>
-    <mergeCell ref="A21:F21"/>
-    <mergeCell ref="A33:O33"/>
-    <mergeCell ref="A34:E34"/>
-    <mergeCell ref="A36:B36"/>
-    <mergeCell ref="A37:B37"/>
-    <mergeCell ref="A22:F22"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>

</xml_diff>